<commit_message>
Register: load council county settlements audit
- 48 sites in 13 Development Plan settlements as 'Council audit - county'; capacity = area x council density
- sites clipped where consents granted since 2022 overlap them; 7 fully covered sites dropped
- interim zoned-land estimates replaced in audited settlements; LAP towns stay on the interim estimate
- validation checks C1-C3 for county audit coverage and changes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -24,7 +24,9 @@
     <sheet name="P7" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="E1" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="E3" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="QA sample" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="C2" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="C3" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="QA sample" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-15 16:21</t>
+          <t>2026-10-23 11:53</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -481,13 +483,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -551,7 +553,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>445 parcels</t>
+          <t>447 parcels</t>
         </is>
       </c>
     </row>
@@ -971,7 +973,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{'Inside catchment': 356, 'Rest of county': 47, 'Zoned in': 28, 'Edge of settlement (within 500 m)': 13, 'Named in scheme, within 2 km': 1}</t>
+          <t>{'Inside catchment': 359, 'Rest of county': 46, 'Zoned in': 28, 'Edge of settlement (within 500 m)': 13, 'Named in scheme, within 2 km': 1}</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1003,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>236 of 242 references found live (15/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
+          <t>236 of 242 references found live (23/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
         </is>
       </c>
     </row>
@@ -1348,12 +1350,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>county settlements audit loaded</t>
+          <t>county audit loaded; no interim zoned-land parcel overlaps it</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>WARN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -1361,7 +1363,67 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>not yet received; 124 interim zoned-land parcels (3,507 homes) stand in for it</t>
+          <t>41 county audit parcels, 728 homes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>County audit</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>county settlements still on interim zoning estimates (not in the council audit)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>83</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2,758 homes in 9 plan areas: ask the council for audits of these towns</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>County audit</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>county audit sites changed on loading (clipped by later consents, or no density given)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>WARN</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>7</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>the audit was drawn for the 2022 plan; consents granted since keep their own land</t>
         </is>
       </c>
     </row>
@@ -3774,2054 +3836,456 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>perm_id</t>
+          <t>plan_name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>parcel_id</t>
+          <t>parcels</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>planning_ref</t>
+          <t>ha</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>scheme</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>units</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>status_source</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>mix_source</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>catchment</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>register_link</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>units correct (Y/N)</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>status correct (Y/N)</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>location correct (Y/N)</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>checked by</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>note</t>
+          <t>homes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>998747</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>PC-188007</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>188007</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">€8.9m - Residential Development </t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>43</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Register description</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Southhill</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/188007/0</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+          <t>Abbeyfeale Local Area PLan 2023-2029</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8.481999999999999</v>
+      </c>
+      <c r="D2" t="n">
+        <v>176</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1045778</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>PC-181193</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>19444</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">€2.2m - Housing Development </t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>GeoDirectory 2026-06-09</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Not available (no bedroom detail in register text)</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Patrickswell</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/19444/0</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+          <t>Adare Local Area Plan 2024-2030</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9.208</v>
+      </c>
+      <c r="D3" t="n">
+        <v>191</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1144674</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PC-2148</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2148</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>€1.9m - Change of Use to 9 Apartments, St. Paul's Convent</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Register description</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Kilfinnane</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2148/0</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+          <t>Caherconlish Local Area Plan 2023-2029</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.792</v>
+      </c>
+      <c r="D4" t="n">
+        <v>190</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1164066</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PC-21550</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>21550</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">€1.9m - 9 Houses </t>
-        </is>
-      </c>
-      <c r="E5" t="n">
+          <t>Castleconnell Local Area Plan 2023-2029</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>9</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Not available (no bedroom detail in register text)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Caherconlish</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/21550/0</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="C5" t="n">
+        <v>10.119</v>
+      </c>
+      <c r="D5" t="n">
+        <v>208</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1010675</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>PC-ABPREF307631</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>187031</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>€11m - Residential Development, Castletroy</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>54</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>GeoDirectory 2026-06-09</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Not available (register text incomplete)</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Castletroy/Annacotty</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/187031/0</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+          <t>Croom Local Area Plan 2020-2026</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>9.170999999999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>192</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1024750</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>PC-181243</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>181243</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>€6.4m - Residential Development, Crossagalla</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>53</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Not available (no bedroom detail in register text)</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Southhill</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/181243/0</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+          <t>Kilmallock Local Area Plan 2019-2025</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" t="n">
+        <v>17.391</v>
+      </c>
+      <c r="D7" t="n">
+        <v>355</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>895586</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>PC-191060</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>191060</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>€50m - 1 BQ Development, Limerick City</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Not available (no bedroom detail in register text)</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>City Centre</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/191060/0</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+          <t>Newcastle West Local Area Plan 2023-2029</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>19</v>
+      </c>
+      <c r="C8" t="n">
+        <v>53.032</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1179</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1015929</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>PC-CIS1015929</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">€2m - Housing Development </t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>17</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Expired – not started</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Not available (not in register)</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Rest of county</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+          <t>Patrickswell Local Area Plan 2024-2030</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="D9" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1446285</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>PC-21594</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2660232</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>€7.8m - Residential Development, Abbeyfeale</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>48</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>In planning</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Register description</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Abbeyfeale</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2660232/0</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>1419614</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>CITY-41</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>258327</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>€4.8m - Apartment Development, Limerick</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>30</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>In planning</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>CIS / KPMG</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Kings Island</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/258327/0</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>1428325</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>CITY-72</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2660275</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>€42m - Large Residential Development,Limerick</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>212</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>CIS / KPMG</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Castletroy/Annacotty</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2660275/0</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>1148944</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>PC-21147</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>21147</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">€1.4m - Housing Development </t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>11</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Not available (no bedroom detail in register text)</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Caherdavin</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/21147/0</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>1254537</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>PC-221107</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>221107</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>€5m - Apartment/Retail Development, Dooradoyle</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>30</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>CIS / KPMG</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Dooradoyle</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/221107/0</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>1214059</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>CITY-1</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>ABPREF312683</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>€27.5m - Clonmacken Gardens Housing Development, Limerick</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>165</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>CIS / KPMG</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Caherdavin</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>1409292</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>PC-2560595</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2560595</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>€819k - 6 Apartments</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>6</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Register description</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>City Centre</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560595/0</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>1071780</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>PC-198009</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>198009</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">€1.8m - Housing Development </t>
-        </is>
-      </c>
-      <c r="E17" t="n">
+          <t>Rathkeale Local Area Plan 2023-2029</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" t="n">
+        <v>8.846</v>
+      </c>
+      <c r="D10" t="n">
+        <v>189</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>parcel_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>local_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>zoning</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>developable_area_ha</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>capacity_used</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>capacity_basis</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CTY-BRUFF-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bruff – site 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.332</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>clipped by consent 2360794</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CTY-BRUFF-3</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bruff – site 3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>clipped by consent 2560947</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CTY-CAPPAMORE-1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cappamore – site 1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.5620000000000001</v>
+      </c>
+      <c r="E4" t="n">
         <v>12</v>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Register description</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Rest of county</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/198009/0</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>1412002</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>CITY-91</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2560780</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>€95m - Dock Road LRD, Limerick</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>285</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>CIS / KPMG</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>City Centre</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560780/0</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>1393371</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>CITY-83</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>2560169</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>€4.8m - Mixed Use Development, Limerick</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>30</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>CIS / KPMG</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Singland/Garryowen</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560169/0</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>1446288</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>CITY-57</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>2660241</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>€125.6m - Large Residential Development, Castletroy</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>523</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Register description</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Castletroy/Annacotty</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2660241/0</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>1328561</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>PC-2460046</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>2460046</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>€2m - 7 Houses, Broadford</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>7</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Register description</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Rest of county</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2460046/0</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>1409934</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>PC-2560156</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>2560653</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>€9.4m - Residential Development</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>40</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Stalled</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Planning file documents</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Patrickswell</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560653/0</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>1395070</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>PC-2560211</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>2560211</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">€800k - 4 Apartments </t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>4</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Not available (no bedroom detail in register text)</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Moroe</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560211/0</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>1417511</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>PC-2561228</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>2561228</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>€18.4m - Residential Development, Patrickswell</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>54</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Register description</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Patrickswell</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2561228/0</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>1327848</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>CITY-5</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>2460032</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>€18.9m - Residential Development, Old Cratloe Road</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>99</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>CIS / KPMG</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Caherdavin</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2460032/0</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>1384661</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>PC-2560001</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>2560001</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>€1.3m - 6 Apartments, Thomondgate</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>7</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Not available (no bedroom detail in register text)</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>City Centre</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560001/0</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>1203836</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>PC-218012</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>218012</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>€2.4m - Residential Development</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>18</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Register description</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Rest of county</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/218012/0</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>1063948</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>PC-Part81063948</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Part 8 - 1063948</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>€9m - Rapid Housing Delivery</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>38</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Not available (not in register)</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Caherdavin</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>1350850</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>PC-2460568</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>2460568</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>€3.9m - Residential Development, Castlemahon</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>18</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Not available (no bedroom detail in register text)</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Rest of county</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2460568/0</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>1278374</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>PC-2360150</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>2360150</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>€3m - Apartment Development, Limerick</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>24</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>CIS / KPMG</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>City Centre</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2360150/0</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>1193936</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>PC-211152</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>211400</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>€21m - Newtow Meadows Development, Phase 4, Castletroy</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>98</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>CIS / KPMG</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Castletroy/Annacotty</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>CIS</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/211400/0</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>REG-178015</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>PC-178015</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>178015</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Part 8: provision of 5 no. residential terraced units (all two storey) and all</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>5</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>GeoDirectory 2026-06-09</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Not available</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Southhill</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>Register only (Part 8, not in CIS)</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/178015/0</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>REG-24151</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>PC-24151</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>24151</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Register: the construction of 10 dwelling units to include 2 no. detached 5 bedr</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>10</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Permitted – not started</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Not available</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Croom</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Register only (private, not in CIS)</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/24151/0</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>REG-188012</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>PC-228017</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>188012</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Part 8: (a) provision of 24 no. two storey residential housing units. The unit</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>24</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Under construction</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>CIS / building control</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Not available</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Patrickswell</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Register only (Part 8, not in CIS)</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/188012/0</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>clipped by consent 221352</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CTY-CAPPAMORE-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Cappamore – site 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>clipped by consent 19872</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CTY-HOSPITAL-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Hospital – site 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Enterprise &amp; Employment</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2.675</v>
+      </c>
+      <c r="E6" t="n">
+        <v>67</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Estimate (council audit recorded no capacity): developable area x density</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>County audit gives no density; zoned Enterprise &amp; Employment</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CTY-KILFINANE-1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Kilfinane – site 1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>clipped by consent 218013</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CTY-PALLASKENRY-4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pallaskenry – site 4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>clipped by consent 24352</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5908,6 +4372,2066 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>perm_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>parcel_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>planning_ref</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>scheme</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>units</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>status_source</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>mix_source</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>catchment</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>register_link</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>units correct (Y/N)</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>status correct (Y/N)</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>location correct (Y/N)</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>checked by</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>998747</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PC-188007</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>188007</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€8.9m - Residential Development </t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>43</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Register description</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Southhill</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/188007/0</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1045778</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PC-181193</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>19444</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€2.2m - Housing Development </t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>GeoDirectory 2026-06-09</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Not available (no bedroom detail in register text)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Patrickswell</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/19444/0</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1144674</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PC-2148</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2148</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>€1.9m - Change of Use to 9 Apartments, St. Paul's Convent</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Register description</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Kilfinnane</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2148/0</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1164066</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PC-21550</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>21550</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€1.9m - 9 Houses </t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>9</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Not available (no bedroom detail in register text)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Caherconlish</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/21550/0</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1010675</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PC-ABPREF307631</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>187031</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>€11m - Residential Development, Castletroy</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>54</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>GeoDirectory 2026-06-09</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Not available (register text incomplete)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Castletroy/Annacotty</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/187031/0</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1024750</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PC-181243</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>181243</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>€6.4m - Residential Development, Crossagalla</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>53</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Not available (no bedroom detail in register text)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Southhill</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/181243/0</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>895586</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PC-191060</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>191060</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>€50m - 1 BQ Development, Limerick City</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>35</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Not available (no bedroom detail in register text)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>City Centre</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/191060/0</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1015929</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PC-CIS1015929</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€2m - Housing Development </t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>17</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Expired – not started</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Not available (not in register)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Rest of county</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1446285</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PC-21594</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2660232</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>€7.8m - Residential Development, Abbeyfeale</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>48</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>In planning</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Register description</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Abbeyfeale</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2660232/0</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1419614</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CITY-41</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>258327</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>€4.8m - Apartment Development, Limerick</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>In planning</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>CIS / KPMG</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Kings Island</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/258327/0</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1428325</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CITY-72</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2660275</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>€42m - Large Residential Development,Limerick</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>212</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>CIS / KPMG</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Castletroy/Annacotty</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2660275/0</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1148944</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PC-21147</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>21147</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€1.4m - Housing Development </t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Not available (no bedroom detail in register text)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Caherdavin</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/21147/0</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1254537</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PC-221107</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>221107</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>€5m - Apartment/Retail Development, Dooradoyle</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>30</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>CIS / KPMG</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Dooradoyle</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/221107/0</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1214059</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CITY-1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ABPREF312683</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>€27.5m - Clonmacken Gardens Housing Development, Limerick</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>165</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>CIS / KPMG</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Caherdavin</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1409292</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PC-2560595</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2560595</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>€819k - 6 Apartments</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Register description</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>City Centre</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560595/0</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1071780</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PC-198009</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>198009</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€1.8m - Housing Development </t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>12</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Register description</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Rest of county</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/198009/0</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1412002</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CITY-91</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2560780</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>€95m - Dock Road LRD, Limerick</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>285</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>CIS / KPMG</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>City Centre</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560780/0</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1393371</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CITY-83</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2560169</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>€4.8m - Mixed Use Development, Limerick</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>30</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>CIS / KPMG</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Singland/Garryowen</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560169/0</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1446288</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CITY-57</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2660241</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>€125.6m - Large Residential Development, Castletroy</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>523</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Register description</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Castletroy/Annacotty</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2660241/0</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1328561</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PC-2460046</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2460046</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>€2m - 7 Houses, Broadford</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>7</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Register description</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Rest of county</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2460046/0</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1409934</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PC-2560156</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2560653</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>€9.4m - Residential Development</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>40</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Stalled</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Planning file documents</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Patrickswell</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560653/0</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1395070</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PC-2560211</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2560211</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€800k - 4 Apartments </t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Not available (no bedroom detail in register text)</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Moroe</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560211/0</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1417511</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PC-2561228</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2561228</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>€18.4m - Residential Development, Patrickswell</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>54</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Register description</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Patrickswell</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2561228/0</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1327848</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CITY-5</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2460032</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>€18.9m - Residential Development, Old Cratloe Road</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>99</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>CIS / KPMG</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Caherdavin</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2460032/0</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1384661</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PC-2560001</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2560001</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>€1.3m - 6 Apartments, Thomondgate</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Not available (no bedroom detail in register text)</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>City Centre</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2560001/0</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1203836</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PC-218012</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>218012</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>€2.4m - Residential Development</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>18</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Register description</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Rest of county</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/218012/0</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1063948</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PC-Part81063948</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Part 8 - 1063948</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>€9m - Rapid Housing Delivery</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>38</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Not available (not in register)</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Caherdavin</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1350850</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PC-2460568</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2460568</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>€3.9m - Residential Development, Castlemahon</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>18</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Not available (no bedroom detail in register text)</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Rest of county</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2460568/0</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1278374</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PC-2360150</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2360150</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>€3m - Apartment Development, Limerick</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>24</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>CIS / KPMG</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>City Centre</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/2360150/0</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1193936</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PC-211152</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>211400</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>€21m - Newtow Meadows Development, Phase 4, Castletroy</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>98</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>CIS / KPMG</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Castletroy/Annacotty</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/211400/0</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>REG-178015</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PC-178015</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>178015</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Part 8: provision of 5 no. residential terraced units (all two storey) and all</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>GeoDirectory 2026-06-09</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Southhill</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Register only (Part 8, not in CIS)</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/178015/0</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>REG-24151</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PC-24151</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>24151</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Register: the construction of 10 dwelling units to include 2 no. detached 5 bedr</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>10</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Croom</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Register only (private, not in CIS)</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/24151/0</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>REG-188012</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>PC-188012</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>188012</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Part 8: (a) provision of 24 no. two storey residential housing units. The unit</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>24</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Under construction</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>CIS / building control</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Patrickswell</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Register only (Part 8, not in CIS)</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>https://eplanning.ie/LimerickCCC/AppFileRefDetails/188012/0</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Register: merge 'Council audit – reinstated' into 'Council audit'
The three reinstated sites (CITY-2, CITY-35, CITY-112) keep the reason in notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-23 11:53</t>
+          <t>2026-10-26 12:20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>236 of 242 references found live (23/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
+          <t>236 of 242 references found live (26/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: add Askeaton future residential zoning (missing from national GZT file)
9 zoned-land parcels, 23 ha, about 474 homes at local densities; Phase 2 and Red wastewater status noted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-26 12:20</t>
+          <t>2026-10-26 12:45</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>447 parcels</t>
+          <t>456 parcels</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{'Inside catchment': 359, 'Rest of county': 46, 'Zoned in': 28, 'Edge of settlement (within 500 m)': 13, 'Named in scheme, within 2 km': 1}</t>
+          <t>{'Inside catchment': 364, 'Rest of county': 46, 'Zoned in': 32, 'Edge of settlement (within 500 m)': 13, 'Named in scheme, within 2 km': 1}</t>
         </is>
       </c>
     </row>
@@ -1389,11 +1389,11 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2,758 homes in 9 plan areas: ask the council for audits of these towns</t>
+          <t>3,232 homes in 10 plan areas: ask the council for audits of these towns</t>
         </is>
       </c>
     </row>
@@ -3836,7 +3836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3896,112 +3896,128 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Caherconlish Local Area Plan 2023-2029</t>
+          <t>Askeaton Local Area Plan (council zoning file, Oct 2026)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>8.792</v>
+        <v>23.318</v>
       </c>
       <c r="D4" t="n">
-        <v>190</v>
+        <v>474</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Castleconnell Local Area Plan 2023-2029</t>
+          <t>Caherconlish Local Area Plan 2023-2029</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C5" t="n">
-        <v>10.119</v>
+        <v>8.792</v>
       </c>
       <c r="D5" t="n">
-        <v>208</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Croom Local Area Plan 2020-2026</t>
+          <t>Castleconnell Local Area Plan 2023-2029</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>9.170999999999999</v>
+        <v>10.119</v>
       </c>
       <c r="D6" t="n">
-        <v>192</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kilmallock Local Area Plan 2019-2025</t>
+          <t>Croom Local Area Plan 2020-2026</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>17.391</v>
+        <v>9.170999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>355</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Newcastle West Local Area Plan 2023-2029</t>
+          <t>Kilmallock Local Area Plan 2019-2025</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C8" t="n">
-        <v>53.032</v>
+        <v>17.391</v>
       </c>
       <c r="D8" t="n">
-        <v>1179</v>
+        <v>355</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Patrickswell Local Area Plan 2024-2030</t>
+          <t>Newcastle West Local Area Plan 2023-2029</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C9" t="n">
-        <v>3.49</v>
+        <v>53.032</v>
       </c>
       <c r="D9" t="n">
-        <v>78</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Patrickswell Local Area Plan 2024-2030</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="D10" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Rathkeale Local Area Plan 2023-2029</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
         <v>10</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C11" t="n">
         <v>8.846</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>189</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: county audit from council Excel (May 2026) placed on polygons
- 126 Excel sites matched to zoning polygons; 90 placed (confirmed or high confidence), 34 listed for manual placement
- all council-supplied polygons included; unmatched ones carry no capacity until filled in
- 2022 audit kept for the 8 settlements the Excel omits; council zero capacities respected

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-26 12:45</t>
+          <t>2026-10-26 14:58</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>456 parcels</t>
+          <t>457 parcels</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{'Inside catchment': 364, 'Rest of county': 46, 'Zoned in': 32, 'Edge of settlement (within 500 m)': 13, 'Named in scheme, within 2 km': 1}</t>
+          <t>{'Inside catchment': 367, 'Rest of county': 46, 'Edge of settlement (within 500 m)': 34, 'Zoned in': 9, 'Named in scheme, within 2 km': 1}</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>41 county audit parcels, 728 homes</t>
+          <t>116 county audit parcels, 2,832 homes</t>
         </is>
       </c>
     </row>
@@ -1389,11 +1389,11 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>3,232 homes in 10 plan areas: ask the council for audits of these towns</t>
+          <t>1,120 homes in 8 plan areas: ask the council for audits of these towns</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>116</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -3836,7 +3836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3868,13 +3868,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>8.481999999999999</v>
+        <v>2.102</v>
       </c>
       <c r="D2" t="n">
-        <v>176</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
@@ -3884,141 +3884,109 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>9.208</v>
+        <v>5.959</v>
       </c>
       <c r="D3" t="n">
-        <v>191</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Askeaton Local Area Plan (council zoning file, Oct 2026)</t>
+          <t>Caherconlish Local Area Plan 2023-2029</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>23.318</v>
+        <v>2.578</v>
       </c>
       <c r="D4" t="n">
-        <v>474</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Caherconlish Local Area Plan 2023-2029</t>
+          <t>Castleconnell Local Area Plan 2023-2029</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>8.792</v>
+        <v>1.653</v>
       </c>
       <c r="D5" t="n">
-        <v>190</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Castleconnell Local Area Plan 2023-2029</t>
+          <t>Croom Local Area Plan 2020-2026</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>10.119</v>
+        <v>0.193</v>
       </c>
       <c r="D6" t="n">
-        <v>208</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Croom Local Area Plan 2020-2026</t>
+          <t>Kilmallock Local Area Plan 2019-2025</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>9.170999999999999</v>
+        <v>0.947</v>
       </c>
       <c r="D7" t="n">
-        <v>192</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kilmallock Local Area Plan 2019-2025</t>
+          <t>Newcastle West Local Area Plan 2023-2029</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>17.391</v>
+        <v>37.599</v>
       </c>
       <c r="D8" t="n">
-        <v>355</v>
+        <v>827</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Newcastle West Local Area Plan 2023-2029</t>
+          <t>Patrickswell Local Area Plan 2024-2030</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>53.032</v>
+        <v>0.384</v>
       </c>
       <c r="D9" t="n">
-        <v>1179</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Patrickswell Local Area Plan 2024-2030</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
         <v>9</v>
-      </c>
-      <c r="C10" t="n">
-        <v>3.49</v>
-      </c>
-      <c r="D10" t="n">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Rathkeale Local Area Plan 2023-2029</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="n">
-        <v>8.846</v>
-      </c>
-      <c r="D11" t="n">
-        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -4032,7 +4000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4075,231 +4043,3760 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-1</t>
+          <t>CTY-NEWCASTLEWES-2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bruff – site 1</t>
+          <t>Newcastle West – site 2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Town Centre</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.332</v>
+        <v>0.4</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Council county audit: area x density</t>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>clipped by consent 2360794</t>
+          <t>Site status: No Permission; Pre Planning - 16761 - 24 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-3</t>
+          <t>CTY-NEWCASTLEWES-5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bruff – site 3</t>
+          <t>Newcastle West – site 5</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.377</v>
+        <v>12.5</v>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>438</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Council county audit: area x density</t>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>clipped by consent 2560947</t>
+          <t>Site status: Partially Development - Reduced Area Available; Permission: 22840 - 93 units; Is part of this built out?; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-1</t>
+          <t>CTY-NEWCASTLEWES-6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cappamore – site 1</t>
+          <t>Newcastle West – site 6</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.238</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Council county audit: area x density</t>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>clipped by consent 221352</t>
+          <t>Site status: Partially Development - Reduced Area Available; Permission: 2360706 - 53 units, 17383 - 54 units; Placement: area match (High); clipped by consent 2360706</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-4</t>
+          <t>CTY-NEWCASTLEWES-11D</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cappamore – site 4</t>
+          <t>Newcastle West – site 11D</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.063</v>
+        <v>1.38</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Council county audit: area x density</t>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>clipped by consent 19872</t>
+          <t>Site status: No Permission; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-5</t>
+          <t>CTY-NEWCASTLEWES-12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hospital – site 5</t>
+          <t>Newcastle West – site 12</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Enterprise &amp; Employment</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.675</v>
+        <v>0.8</v>
       </c>
       <c r="E6" t="n">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Estimate (council audit recorded no capacity): developable area x density</t>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>County audit gives no density; zoned Enterprise &amp; Employment</t>
+          <t>Site status: No Permission; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-1</t>
+          <t>CTY-NEWCASTLEWES-13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kilfinane – site 1</t>
+          <t>Newcastle West – site 13</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.091</v>
+        <v>2.1</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Council county audit: area x density</t>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>clipped by consent 218013</t>
+          <t>Site status: Permission Granted; Permission: 2360826 - 14 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>CTY-NEWCASTLEWES-14</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Newcastle West – site 14</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.595</v>
+      </c>
+      <c r="E8" t="n">
+        <v>21</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 228020 - P8 21 units; Placement: area match (High); clipped by consent 228020</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CTY-NEWCASTLEWES-17</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Newcastle West – site 17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="E9" t="n">
+        <v>39</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Is this land directly accessible to services?; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CTY-ABBEYFEALE-1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Abbeyfeale – site 1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Town Centre</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E10" t="n">
+        <v>19</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Requires Site Assembly ; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CTY-ABBEYFEALE-3</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Abbeyfeale – site 3</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Town Centre</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Requires Site Assembly ; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CTY-ABBEYFEALE-5</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Abbeyfeale – site 5</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2.017</v>
+      </c>
+      <c r="E12" t="n">
+        <v>44</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 2660232 - 48 unitss, 2.081; 21594 - 68 units, 2.79ha.; 2460606 - 40 units, 1.76ha. Appeal Refused by ACP ; Placement: area match (High); clipped by consent 21594</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CTY-ABBEYFEALE-7</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Abbeyfeale – site 7</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>10</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CTY-ABBEYFEALE-8</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Abbeyfeale – site 8</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E14" t="n">
+        <v>31</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CTY-ABBEYFEALE-9</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Abbeyfeale – site 9</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CTY-ABBEYFEALE-10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Abbeyfeale – site 10</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CTY-CASTLECONNEL-1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Castleconnell – site 1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="E17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CTY-CASTLECONNEL-2</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Castleconnell – site 2</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="E18" t="n">
+        <v>14</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CTY-CASTLECONNEL-3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Castleconnell – site 3</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="E19" t="n">
+        <v>14</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CTY-CASTLECONNEL-4</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Castleconnell – site 4</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2.713</v>
+      </c>
+      <c r="E20" t="n">
+        <v>60</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Site status: Commenced -Reduced area available; Permission: 2360866 - 74 units; Placement: area match (Low), confirmed by analyst; clipped by consent 2360866</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CTY-CASTLECONNEL-5</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Castleconnell – site 5</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E21" t="n">
+        <v>11</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 25327 - 2units; Placement: area match (Medium), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CTY-CASTLECONNEL-6</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Castleconnell – site 6</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>11</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Pre Planning 562893 - 25 units; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CTY-CASTLECONNEL-8</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Castleconnell – site 8</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E23" t="n">
+        <v>16</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CTY-CASTLECONNEL-9</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Castleconnell – site 9</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>4.009</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; on the council map but not in the Excel; 9/10 order to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CTY-CASTLECONNEL-10</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Castleconnell – site 10</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>6.742</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; on the council map but not in the Excel; 9/10 order to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CTY-CAHERCONLISH-1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Caherconlish – site 1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="E26" t="n">
+        <v>79</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Pre Planning 1032260 - 58 units; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CTY-CAHERCONLISH-2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Caherconlish – site 2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0.439</v>
+      </c>
+      <c r="E27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: placed per analyst (council map): west of site 3; two zoning polygons together = 0.44 ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CTY-CAHERCONLISH-3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Caherconlish – site 3</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0.234</v>
+      </c>
+      <c r="E28" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match; confirm (analyst marked the first placement of 3 wrong)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CTY-CAHERCONLISH-5</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Caherconlish – site 5</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2.085</v>
+      </c>
+      <c r="E29" t="n">
+        <v>21</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Pre Planning - 1049863 - 110 units; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CTY-CAHERCONLISH-7</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Caherconlish – site 7</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="n">
+        <v>5.889</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; site 7 is on the council map but not in the Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E31" t="n">
+        <v>9</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: placed per analyst (council map): northwest of site 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1.039</v>
+      </c>
+      <c r="E32" t="n">
+        <v>23</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 3</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="E33" t="n">
+        <v>35</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-4</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 4</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E34" t="n">
+        <v>8</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-5</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 5</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0.601</v>
+      </c>
+      <c r="E35" t="n">
+        <v>13</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-6</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 6</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E36" t="n">
+        <v>18</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: placed per analyst (council map); Excel area 0.82 ha vs polygon 0.38 ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-7</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 7</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="E37" t="n">
+        <v>28</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-8</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 8</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="E38" t="n">
+        <v>30</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-9</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 9</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="E39" t="n">
+        <v>4</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-10</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Rathkeale – site 10</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1.785</v>
+      </c>
+      <c r="E40" t="n">
+        <v>18</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CTY-KILMALLOCK-1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Kilmallock – site 1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Residential Development Area</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>2.782</v>
+      </c>
+      <c r="E41" t="n">
+        <v>61</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Site status: Under Construction; Permission: 2326 - 28 units; Placement: area match (Medium), confirmed by analyst; clipped by consent 2326</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CTY-KILMALLOCK-2</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Kilmallock – site 2</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>3.657</v>
+      </c>
+      <c r="E42" t="n">
+        <v>37</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Pre Planning for 26 units; Placement: area match (Medium), confirmed by analyst; clipped by consent 2326</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CTY-KILMALLOCK-8</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Kilmallock – site 8</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="E43" t="n">
+        <v>37</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CTY-KILMALLOCK-9</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Kilmallock – site 9</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Residential Development Area</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="E44" t="n">
+        <v>117</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Site status: No Permission; Placement: area match (Low), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CTY-KILMALLOCK-10</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Kilmallock – site 10</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Residential Development Area</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>2.967</v>
+      </c>
+      <c r="E45" t="n">
+        <v>65</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Site status: Under Construction; Permission: 2460788 - 42 units on 1.64; Placement: area match (High), confirmed by analyst; clipped by consent 2460788</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>CTY-ADARE-1A</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Adare – site 1a</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 198010 - P8 31 units &amp; 8 plots; Placement: area match (High); clipped by consent 198010; clipped by consent 22990</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CTY-ADARE-5</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Adare – site 5</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E47" t="n">
+        <v>37</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CTY-ADARE-6</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Adare – site 6</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="E48" t="n">
+        <v>7</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CTY-ADARE-8</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Adare – site 8</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E49" t="n">
+        <v>12</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CTY-ASKEATON-6</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Askeaton – site 6</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites - Phase 1</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="E50" t="n">
+        <v>10</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CTY-ASKEATON-10</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Askeaton – site 10</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Residential Development Area - Phase 2</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>4.719</v>
+      </c>
+      <c r="E51" t="n">
+        <v>104</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CTY-ASKEATON-9</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Askeaton – site 9</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites - Phase 2</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>2.459</v>
+      </c>
+      <c r="E52" t="n">
+        <v>25</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CTY-BRUFF-1</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bruff – site 1</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>0.332</v>
+      </c>
+      <c r="E53" t="n">
+        <v>7</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 2360794 - 74 units; Placement: area match (High); clipped by consent 2360794</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CTY-BRUFF-2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bruff – site 2</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0.679</v>
+      </c>
+      <c r="E54" t="n">
+        <v>15</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Site status: Permission Sought; Permission: 24179002 - 18 units on 0.82ha. ; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CTY-BRUFF-4</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Bruff – site 4</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0.234</v>
+      </c>
+      <c r="E55" t="n">
+        <v>5</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 2360796 - 5 units; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CTY-BRUFF-3</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Bruff – site 3</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E56" t="n">
+        <v>14</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 2560947 - 8 units on  0.349; Placement: area match (High); clipped by consent 2560947</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CTY-CAPPAMORE-1</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Cappamore – site 1</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>0.5620000000000001</v>
+      </c>
+      <c r="E57" t="n">
+        <v>12</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Site status: Under Construction; Permission: 221352 - 17 units; Placement: area match (High); clipped by consent 221352</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CTY-CAPPAMORE-2</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Cappamore – site 2</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="E58" t="n">
+        <v>7</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CTY-CAPPAMORE-3</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Cappamore – site 3</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1.012</v>
+      </c>
+      <c r="E59" t="n">
+        <v>22</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Site status: Under Construction; Permission: 23529 - 22 units; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CTY-CAPPAMORE-4</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Cappamore – site 4</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>0.062</v>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Site status: Under Construction; Permission: 19872 - 10 units; Placement: area match (High); clipped by consent 19872</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>CTY-CROOM-1</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Croom – site 1</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Residential Development Area - Phase 1</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="E61" t="n">
+        <v>11</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CTY-CROOM-2</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Croom – site 2</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Residential Development Area - Phase 1</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>2.951</v>
+      </c>
+      <c r="E62" t="n">
+        <v>65</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 21630 - 51 units on 2.007; Reduced site area available due to road construction ; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>CTY-CROOM-3</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Croom – site 3</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites - Phase 1</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0.369</v>
+      </c>
+      <c r="E63" t="n">
+        <v>4</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Site status: Complete; Permission: 21649 - 1 unit, 201219 - 1 unit; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>CTY-CROOM-5</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Croom – site 5</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Residential Development Area - Phase 1</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="E64" t="n">
+        <v>89</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>CTY-CROOM-6</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Croom – site 6</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Residential Development Area - Phase 1</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>2.007</v>
+      </c>
+      <c r="E65" t="n">
+        <v>44</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Site status: Complete; Permission: 22267 - 56 units; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>CTY-CROOM-7</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Croom – site 7</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites - Phase 1</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>2.677</v>
+      </c>
+      <c r="E66" t="n">
+        <v>27</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>CTY-HOSPITAL-1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Hospital – site 1</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>0.627</v>
+      </c>
+      <c r="E67" t="n">
+        <v>14</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Pre Planning 16801 - 21 units; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>CTY-HOSPITAL-2</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Hospital – site 2</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>1.001</v>
+      </c>
+      <c r="E68" t="n">
+        <v>22</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>CTY-HOSPITAL-3</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Hospital – site 3</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="E69" t="n">
+        <v>15</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>CTY-HOSPITAL-4</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Hospital – site 4</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1.019</v>
+      </c>
+      <c r="E70" t="n">
+        <v>10</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>CTY-KILFINANE-1</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Kilfinane – site 1</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Site status: Under Construction; Permission: 218013 - P8 10 units; Under construction; Placement: area match (High); clipped by consent 218013</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>CTY-KILFINANE-2</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Kilfinane – site 2</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="E72" t="n">
+        <v>7</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>CTY-KILFINANE-3</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Kilfinane – site 3</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>0.821</v>
+      </c>
+      <c r="E73" t="n">
+        <v>18</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>CTY-KILFINANE-4</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Kilfinane – site 4</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>0.713</v>
+      </c>
+      <c r="E74" t="n">
+        <v>16</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Site Assembly Required; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>CTY-KILFINANE-5</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Kilfinane – site 5</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>1.547</v>
+      </c>
+      <c r="E75" t="n">
+        <v>15</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>CTY-MURROE-1</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Murroe – site 1</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>1.808</v>
+      </c>
+      <c r="E76" t="n">
+        <v>40</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>CTY-MURROE-2</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Murroe – site 2</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="E77" t="n">
+        <v>22</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>CTY-MURROE-4</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Murroe – site 4</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1.938</v>
+      </c>
+      <c r="E78" t="n">
+        <v>19</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-2</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 2</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>1.534</v>
+      </c>
+      <c r="E79" t="n">
+        <v>34</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High); clipped by consent 18346; clipped by consent 2560156</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-17</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 17</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E80" t="n">
+        <v>4</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Site status: No Permission ; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-3</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 3</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E81" t="n">
+        <v>9</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 2560633 - 6 units  on 0.42; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-8</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 8</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>1.772</v>
+      </c>
+      <c r="E82" t="n">
+        <v>39</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Site status: Permission Granted; Permission: 2360144 - 44 units; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-9</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 9</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="E83" t="n">
+        <v>9</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Site status: Under Construction; Permission: 19444 - 16 units, 181193 - 48 units; Placement: area match (High); clipped by consent 181193; clipped by consent 19444</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-10</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 10</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="E84" t="n">
+        <v>19</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-11</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 11</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>New Resi</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="E85" t="n">
+        <v>8</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Site status: Complete; Permission: 19689 - 8 units; Placement: area match (High)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>CTY-NEWCASTLEWES-U1</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Newcastle West – site U1</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Town Centre</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>3.815</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>CTY-NEWCASTLEWES-U2</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Newcastle West – site U2</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Enterprise and Employment</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>25.055</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-U1</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Rathkeale – site U1</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Enterprise and Employment</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>17.768</v>
+      </c>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-U2</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Rathkeale – site U2</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Enterprise and Employment</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>14.728</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>CTY-RATHKEALE-U3</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Rathkeale – site U3</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Enterprise and Employment</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>12.896</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>CTY-ASKEATON-U1</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Askeaton – site U1</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Resi Service Site Phase 2</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>CTY-ASKEATON-U2</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Askeaton – site U2</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Resi Service Site Phase 1</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>1.182</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>CTY-ASKEATON-U3</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Askeaton – site U3</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Resi Development Area Phase 1</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>CTY-ASKEATON-U4</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Askeaton – site U4</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Resi Development Area Phase 1</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>7.428</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0</v>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>CTY-ASKEATON-U5</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Askeaton – site U5</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Resi Service Site Phase 2</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>2.098</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0</v>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>CTY-ASKEATON-U6</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Askeaton – site U6</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Resi Service Site Phase 1</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>2.684</v>
+      </c>
+      <c r="E96" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>CTY-BALLINGARRY-1</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Ballingarry – site 1</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E97" t="n">
+        <v>38</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>CTY-BALLINGARRY-2</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Ballingarry – site 2</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>1.057</v>
+      </c>
+      <c r="E98" t="n">
+        <v>11</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>CTY-BALLINGARRY-3</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Ballingarry – site 3</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>2.903</v>
+      </c>
+      <c r="E99" t="n">
+        <v>29</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>CTY-BRUREE-1</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Bruree – site 1</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E100" t="n">
+        <v>25</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>CTY-BRUREE-2</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Bruree – site 2</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>0.247</v>
+      </c>
+      <c r="E101" t="n">
+        <v>5</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>CTY-BRUREE-3</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Bruree – site 3</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>0.736</v>
+      </c>
+      <c r="E102" t="n">
+        <v>7</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>CTY-DROMCOLLIHER-1</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Dromcolliher – site 1</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="E103" t="n">
+        <v>18</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>CTY-DROMCOLLIHER-2</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Dromcolliher – site 2</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="E104" t="n">
+        <v>2</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>CTY-DROMCOLLIHER-3</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Dromcolliher – site 3</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>0.845</v>
+      </c>
+      <c r="E105" t="n">
+        <v>19</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>CTY-DROMCOLLIHER-4</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Dromcolliher – site 4</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>0.773</v>
+      </c>
+      <c r="E106" t="n">
+        <v>8</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>CTY-FOYNES-1</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Foynes – site 1</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>3.497</v>
+      </c>
+      <c r="E107" t="n">
+        <v>56</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>CTY-GLIN-1</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Glin – site 1</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Mixed Use</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>1.613</v>
+      </c>
+      <c r="E108" t="n">
+        <v>36</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>CTY-GLIN-2</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Glin – site 2</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="E109" t="n">
+        <v>12</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>CTY-GLIN-3</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Glin – site 3</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="E110" t="n">
+        <v>10</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>CTY-GLIN-4</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Glin – site 4</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E111" t="n">
+        <v>27</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>CTY-HOSPITAL-5</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Hospital – site 5</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Enterprise &amp; Employment</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>2.675</v>
+      </c>
+      <c r="E112" t="n">
+        <v>67</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Estimate (council audit recorded no capacity): developable area x density</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>CTY-PALLASGREEN-2</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Pallasgreen – site 2</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>1.424</v>
+      </c>
+      <c r="E113" t="n">
+        <v>31</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>CTY-PALLASGREEN-1</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Pallasgreen – site 1</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>0.613</v>
+      </c>
+      <c r="E114" t="n">
+        <v>14</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>CTY-PALLASGREEN-3</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Pallasgreen – site 3</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E115" t="n">
+        <v>11</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
           <t>CTY-PALLASKENRY-4</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B116" t="inlineStr">
         <is>
           <t>Pallaskenry – site 4</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C116" t="inlineStr">
         <is>
           <t>Residential Serviced Sites</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D116" t="n">
         <v>0.271</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E116" t="n">
         <v>3</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>clipped by consent 24352</t>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon; clipped by consent 24352</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>CTY-PALLASKENRY-3</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Pallaskenry – site 3</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>0.753</v>
+      </c>
+      <c r="E117" t="n">
+        <v>17</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
         </is>
       </c>
     </row>
@@ -6391,7 +9888,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PC-188012</t>
+          <t>PC-228017</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -6538,7 +10035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6637,6 +10134,37 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>Council estimate (area × density band)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CTY-NEWCASTLEWES-6</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Council audit – county</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Newcastle West – site 6</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.238</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
     </row>
@@ -6651,7 +10179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6922,6 +10450,24 @@
       </c>
       <c r="D15" t="n">
         <v>250</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-11</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 11</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Register: keep 2026 council county sites whole; attach permissions mostly inside them
Clipping by later consents now applies only to the 2022 audit sites.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-26 14:58</t>
+          <t>2026-10-26 15:12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>457 parcels</t>
+          <t>448 parcels</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{'Inside catchment': 367, 'Rest of county': 46, 'Edge of settlement (within 500 m)': 34, 'Zoned in': 9, 'Named in scheme, within 2 km': 1}</t>
+          <t>{'Inside catchment': 361, 'Rest of county': 46, 'Edge of settlement (within 500 m)': 31, 'Zoned in': 9, 'Named in scheme, within 2 km': 1}</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>116 county audit parcels, 2,832 homes</t>
+          <t>125 county audit parcels, 3,486 homes</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -3967,7 +3967,7 @@
         <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>37.599</v>
+        <v>37.606</v>
       </c>
       <c r="D8" t="n">
         <v>827</v>
@@ -4000,7 +4000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4123,7 +4123,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.238</v>
+        <v>1.5</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -4135,19 +4135,19 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Site status: Partially Development - Reduced Area Available; Permission: 2360706 - 53 units, 17383 - 54 units; Placement: area match (High); clipped by consent 2360706</t>
+          <t>Site status: Partially Development - Reduced Area Available; Permission: 2360706 - 53 units, 17383 - 54 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-11D</t>
+          <t>CTY-NEWCASTLEWES-8</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Newcastle West – site 11D</t>
+          <t>Newcastle West – site 8</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4156,10 +4156,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.38</v>
+        <v>0.4</v>
       </c>
       <c r="E5" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -4168,19 +4168,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (High)</t>
+          <t>Site status: Permission Sought; Permission: 2660575 - 30 units, 0.428ha. - FI; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-12</t>
+          <t>CTY-NEWCASTLEWES-11D</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Newcastle West – site 12</t>
+          <t>Newcastle West – site 11D</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4189,10 +4189,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.8</v>
+        <v>1.38</v>
       </c>
       <c r="E6" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -4208,12 +4208,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-13</t>
+          <t>CTY-NEWCASTLEWES-12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Newcastle West – site 13</t>
+          <t>Newcastle West – site 12</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4222,10 +4222,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2.1</v>
+        <v>0.8</v>
       </c>
       <c r="E7" t="n">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -4234,19 +4234,19 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2360826 - 14 units; Placement: area match (High)</t>
+          <t>Site status: No Permission; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-14</t>
+          <t>CTY-NEWCASTLEWES-13</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Newcastle West – site 14</t>
+          <t>Newcastle West – site 13</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4255,10 +4255,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.595</v>
+        <v>2.1</v>
       </c>
       <c r="E8" t="n">
-        <v>21</v>
+        <v>74</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -4267,19 +4267,19 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 228020 - P8 21 units; Placement: area match (High); clipped by consent 228020</t>
+          <t>Site status: Permission Granted; Permission: 2360826 - 14 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-17</t>
+          <t>CTY-NEWCASTLEWES-14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Newcastle West – site 17</t>
+          <t>Newcastle West – site 14</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4288,10 +4288,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.12</v>
+        <v>1.3</v>
       </c>
       <c r="E9" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -4300,31 +4300,31 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Is this land directly accessible to services?; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 228020 - P8 21 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-1</t>
+          <t>CTY-NEWCASTLEWES-17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 1</t>
+          <t>Newcastle West – site 17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Town Centre</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.57</v>
+        <v>1.12</v>
       </c>
       <c r="E10" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -4333,19 +4333,19 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Requires Site Assembly ; Placement: area match (High)</t>
+          <t>Site status: No Permission; Is this land directly accessible to services?; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-3</t>
+          <t>CTY-ABBEYFEALE-1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 3</t>
+          <t>Abbeyfeale – site 1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4354,10 +4354,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.26</v>
+        <v>0.57</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -4373,24 +4373,24 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-5</t>
+          <t>CTY-ABBEYFEALE-3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 5</t>
+          <t>Abbeyfeale – site 3</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Town Centre</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2.017</v>
+        <v>0.26</v>
       </c>
       <c r="E12" t="n">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4399,31 +4399,31 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2660232 - 48 unitss, 2.081; 21594 - 68 units, 2.79ha.; 2460606 - 40 units, 1.76ha. Appeal Refused by ACP ; Placement: area match (High); clipped by consent 21594</t>
+          <t>Site status: No Permission; Requires Site Assembly ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-7</t>
+          <t>CTY-ABBEYFEALE-5</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 7</t>
+          <t>Abbeyfeale – site 5</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>92</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -4432,31 +4432,31 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2660232 - 48 unitss, 2.081; 21594 - 68 units, 2.79ha.; 2460606 - 40 units, 1.76ha. Appeal Refused by ACP ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-8</t>
+          <t>CTY-ABBEYFEALE-7</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 8</t>
+          <t>Abbeyfeale – site 7</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -4472,24 +4472,24 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-9</t>
+          <t>CTY-ABBEYFEALE-8</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 9</t>
+          <t>Abbeyfeale – site 8</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E15" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -4505,12 +4505,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-10</t>
+          <t>CTY-ABBEYFEALE-9</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 10</t>
+          <t>Abbeyfeale – site 9</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -4519,10 +4519,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -4538,24 +4538,24 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-1</t>
+          <t>CTY-ABBEYFEALE-10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Castleconnell – site 1</t>
+          <t>Abbeyfeale – site 10</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.26</v>
+        <v>0.5</v>
       </c>
       <c r="E17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4564,19 +4564,19 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-2</t>
+          <t>CTY-CASTLECONNEL-1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Castleconnell – site 2</t>
+          <t>Castleconnell – site 1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -4585,10 +4585,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.63</v>
+        <v>0.26</v>
       </c>
       <c r="E18" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4604,12 +4604,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-3</t>
+          <t>CTY-CASTLECONNEL-2</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Castleconnell – site 3</t>
+          <t>Castleconnell – site 2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4618,7 +4618,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="E19" t="n">
         <v>14</v>
@@ -4637,12 +4637,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-4</t>
+          <t>CTY-CASTLECONNEL-3</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Castleconnell – site 4</t>
+          <t>Castleconnell – site 3</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4651,10 +4651,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2.713</v>
+        <v>0.62</v>
       </c>
       <c r="E20" t="n">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4663,19 +4663,19 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Site status: Commenced -Reduced area available; Permission: 2360866 - 74 units; Placement: area match (Low), confirmed by analyst; clipped by consent 2360866</t>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-5</t>
+          <t>CTY-CASTLECONNEL-4</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Castleconnell – site 5</t>
+          <t>Castleconnell – site 4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4684,10 +4684,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.49</v>
+        <v>6.1</v>
       </c>
       <c r="E21" t="n">
-        <v>11</v>
+        <v>134</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -4696,28 +4696,28 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 25327 - 2units; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: Commenced -Reduced area available; Permission: 2360866 - 74 units; Placement: area match (Low), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-6</t>
+          <t>CTY-CASTLECONNEL-5</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Castleconnell – site 6</t>
+          <t>Castleconnell – site 5</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1.1</v>
+        <v>0.49</v>
       </c>
       <c r="E22" t="n">
         <v>11</v>
@@ -4729,19 +4729,19 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Pre Planning 562893 - 25 units; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Permission Granted; Permission: 25327 - 2units; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-8</t>
+          <t>CTY-CASTLECONNEL-6</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Castleconnell – site 8</t>
+          <t>Castleconnell – site 6</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4750,10 +4750,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="E23" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -4762,49 +4762,57 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: No Permission; Pre Planning 562893 - 25 units; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-9</t>
+          <t>CTY-CASTLECONNEL-8</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Castleconnell – site 9</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+          <t>Castleconnell – site 8</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
       <c r="D24" t="n">
-        <v>4.009</v>
+        <v>1.6</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
+        <v>16</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; on the council map but not in the Excel; 9/10 order to confirm</t>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-10</t>
+          <t>CTY-CASTLECONNEL-9</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Castleconnell – site 10</t>
+          <t>Castleconnell – site 9</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="n">
-        <v>6.742</v>
+        <v>4.009</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -4819,45 +4827,37 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-1</t>
+          <t>CTY-CASTLECONNEL-10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Caherconlish – site 1</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>New Resi</t>
-        </is>
-      </c>
+          <t>Castleconnell – site 10</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>3.58</v>
+        <v>6.742</v>
       </c>
       <c r="E26" t="n">
-        <v>79</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Pre Planning 1032260 - 58 units; Placement: area match (High), confirmed by analyst</t>
+          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; on the council map but not in the Excel; 9/10 order to confirm</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-2</t>
+          <t>CTY-CAHERCONLISH-1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Caherconlish – site 2</t>
+          <t>Caherconlish – site 1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4866,10 +4866,10 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.439</v>
+        <v>3.58</v>
       </c>
       <c r="E27" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -4878,19 +4878,19 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: placed per analyst (council map): west of site 3; two zoning polygons together = 0.44 ha</t>
+          <t>Site status: No Permission; Pre Planning 1032260 - 58 units; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-3</t>
+          <t>CTY-CAHERCONLISH-2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Caherconlish – site 3</t>
+          <t>Caherconlish – site 2</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4899,10 +4899,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.234</v>
+        <v>0.439</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -4911,31 +4911,31 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match; confirm (analyst marked the first placement of 3 wrong)</t>
+          <t>Site status: No Permission; Placement: placed per analyst (council map): west of site 3; two zoning polygons together = 0.44 ha</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-5</t>
+          <t>CTY-CAHERCONLISH-3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Caherconlish – site 5</t>
+          <t>Caherconlish – site 3</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2.085</v>
+        <v>0.234</v>
       </c>
       <c r="E29" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -4944,77 +4944,77 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Pre Planning - 1049863 - 110 units; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: area match; confirm (analyst marked the first placement of 3 wrong)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-7</t>
+          <t>CTY-CAHERCONLISH-5</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Caherconlish – site 7</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>Caherconlish – site 5</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
       <c r="D30" t="n">
-        <v>5.889</v>
+        <v>2.085</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; site 7 is on the council map but not in the Excel</t>
+          <t>Site status: No Permission; Pre Planning - 1049863 - 110 units; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-1</t>
+          <t>CTY-CAHERCONLISH-7</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Rathkeale – site 1</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>New Resi</t>
-        </is>
-      </c>
+          <t>Caherconlish – site 7</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="n">
-        <v>0.4</v>
+        <v>5.889</v>
       </c>
       <c r="E31" t="n">
-        <v>9</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: placed per analyst (council map): northwest of site 2</t>
+          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; site 7 is on the council map but not in the Excel</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-2</t>
+          <t>CTY-RATHKEALE-1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Rathkeale – site 2</t>
+          <t>Rathkeale – site 1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -5023,10 +5023,10 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1.039</v>
+        <v>0.4</v>
       </c>
       <c r="E32" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -5035,19 +5035,19 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: placed per analyst (council map): northwest of site 2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-3</t>
+          <t>CTY-RATHKEALE-2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Rathkeale – site 3</t>
+          <t>Rathkeale – site 2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5056,10 +5056,10 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1.57</v>
+        <v>1.039</v>
       </c>
       <c r="E33" t="n">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -5075,12 +5075,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-4</t>
+          <t>CTY-RATHKEALE-3</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Rathkeale – site 4</t>
+          <t>Rathkeale – site 3</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5089,10 +5089,10 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.36</v>
+        <v>1.57</v>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -5108,12 +5108,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-5</t>
+          <t>CTY-RATHKEALE-4</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Rathkeale – site 5</t>
+          <t>Rathkeale – site 4</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5122,10 +5122,10 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.601</v>
+        <v>0.36</v>
       </c>
       <c r="E35" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -5141,12 +5141,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-6</t>
+          <t>CTY-RATHKEALE-5</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Rathkeale – site 6</t>
+          <t>Rathkeale – site 5</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5155,10 +5155,10 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.82</v>
+        <v>0.601</v>
       </c>
       <c r="E36" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -5167,19 +5167,19 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: placed per analyst (council map); Excel area 0.82 ha vs polygon 0.38 ha</t>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-7</t>
+          <t>CTY-RATHKEALE-6</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Rathkeale – site 7</t>
+          <t>Rathkeale – site 6</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5188,10 +5188,10 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.27</v>
+        <v>0.82</v>
       </c>
       <c r="E37" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -5200,19 +5200,19 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: placed per analyst (council map); Excel area 0.82 ha vs polygon 0.38 ha</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-8</t>
+          <t>CTY-RATHKEALE-7</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Rathkeale – site 8</t>
+          <t>Rathkeale – site 7</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5221,10 +5221,10 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.35</v>
+        <v>1.27</v>
       </c>
       <c r="E38" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -5240,24 +5240,24 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-9</t>
+          <t>CTY-RATHKEALE-8</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Rathkeale – site 9</t>
+          <t>Rathkeale – site 8</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.427</v>
+        <v>1.35</v>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -5273,12 +5273,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-10</t>
+          <t>CTY-RATHKEALE-9</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Rathkeale – site 10</t>
+          <t>Rathkeale – site 9</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -5287,10 +5287,10 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1.785</v>
+        <v>0.427</v>
       </c>
       <c r="E40" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -5306,24 +5306,24 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-1</t>
+          <t>CTY-RATHKEALE-10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Kilmallock – site 1</t>
+          <t>Rathkeale – site 10</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Residential Development Area</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2.782</v>
+        <v>1.785</v>
       </c>
       <c r="E41" t="n">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -5332,31 +5332,31 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 2326 - 28 units; Placement: area match (Medium), confirmed by analyst; clipped by consent 2326</t>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-2</t>
+          <t>CTY-KILMALLOCK-1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Kilmallock – site 2</t>
+          <t>Kilmallock – site 1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>Residential Development Area</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3.657</v>
+        <v>3.88</v>
       </c>
       <c r="E42" t="n">
-        <v>37</v>
+        <v>85</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -5365,19 +5365,19 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Pre Planning for 26 units; Placement: area match (Medium), confirmed by analyst; clipped by consent 2326</t>
+          <t>Site status: Under Construction; Permission: 2326 - 28 units; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-8</t>
+          <t>CTY-KILMALLOCK-2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Kilmallock – site 8</t>
+          <t>Kilmallock – site 2</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5386,10 +5386,10 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3.73</v>
+        <v>3.79</v>
       </c>
       <c r="E43" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -5398,31 +5398,31 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: No Permission; Pre Planning for 26 units; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-9</t>
+          <t>CTY-KILMALLOCK-8</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Kilmallock – site 9</t>
+          <t>Kilmallock – site 8</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Residential Development Area</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>5.33</v>
+        <v>3.73</v>
       </c>
       <c r="E44" t="n">
-        <v>117</v>
+        <v>37</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -5431,19 +5431,19 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (Low), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-10</t>
+          <t>CTY-KILMALLOCK-9</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Kilmallock – site 10</t>
+          <t>Kilmallock – site 9</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5452,10 +5452,10 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2.967</v>
+        <v>5.33</v>
       </c>
       <c r="E45" t="n">
-        <v>65</v>
+        <v>117</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -5464,31 +5464,31 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 2460788 - 42 units on 1.64; Placement: area match (High), confirmed by analyst; clipped by consent 2460788</t>
+          <t>Site status: No Permission; Placement: area match (Low), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CTY-ADARE-1A</t>
+          <t>CTY-KILMALLOCK-10</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Adare – site 1a</t>
+          <t>Kilmallock – site 10</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Development Area</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.104</v>
+        <v>4.24</v>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -5497,19 +5497,19 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 198010 - P8 31 units &amp; 8 plots; Placement: area match (High); clipped by consent 198010; clipped by consent 22990</t>
+          <t>Site status: Under Construction; Permission: 2460788 - 42 units on 1.64; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CTY-ADARE-5</t>
+          <t>CTY-ADARE-1A</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Adare – site 5</t>
+          <t>Adare – site 1a</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5518,10 +5518,10 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="E47" t="n">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -5530,19 +5530,19 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 198010 - P8 31 units &amp; 8 plots; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CTY-ADARE-6</t>
+          <t>CTY-ADARE-5</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Adare – site 6</t>
+          <t>Adare – site 5</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5551,10 +5551,10 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.338</v>
+        <v>1.7</v>
       </c>
       <c r="E48" t="n">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -5570,24 +5570,24 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CTY-ADARE-8</t>
+          <t>CTY-ADARE-6</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Adare – site 8</t>
+          <t>Adare – site 6</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1.15</v>
+        <v>0.338</v>
       </c>
       <c r="E49" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -5603,24 +5603,24 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-6</t>
+          <t>CTY-ADARE-8</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Askeaton – site 6</t>
+          <t>Adare – site 8</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites - Phase 1</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.018</v>
+        <v>1.15</v>
       </c>
       <c r="E50" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -5636,24 +5636,24 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-10</t>
+          <t>CTY-ASKEATON-6</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Askeaton – site 10</t>
+          <t>Askeaton – site 6</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Residential Development Area - Phase 2</t>
+          <t>Residential Serviced Sites - Phase 1</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>4.719</v>
+        <v>1.018</v>
       </c>
       <c r="E51" t="n">
-        <v>104</v>
+        <v>10</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -5669,24 +5669,24 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-9</t>
+          <t>CTY-ASKEATON-10</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Askeaton – site 9</t>
+          <t>Askeaton – site 10</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites - Phase 2</t>
+          <t>Residential Development Area - Phase 2</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2.459</v>
+        <v>4.719</v>
       </c>
       <c r="E52" t="n">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -5702,24 +5702,24 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-1</t>
+          <t>CTY-ASKEATON-9</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Bruff – site 1</t>
+          <t>Askeaton – site 9</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites - Phase 2</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.332</v>
+        <v>2.459</v>
       </c>
       <c r="E53" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -5728,19 +5728,19 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2360794 - 74 units; Placement: area match (High); clipped by consent 2360794</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-2</t>
+          <t>CTY-BRUFF-1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Bruff – site 2</t>
+          <t>Bruff – site 1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -5749,10 +5749,10 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.679</v>
+        <v>3.277</v>
       </c>
       <c r="E54" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -5761,19 +5761,19 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Site status: Permission Sought; Permission: 24179002 - 18 units on 0.82ha. ; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2360794 - 74 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-4</t>
+          <t>CTY-BRUFF-2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Bruff – site 4</t>
+          <t>Bruff – site 2</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -5782,10 +5782,10 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.234</v>
+        <v>0.679</v>
       </c>
       <c r="E55" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -5794,31 +5794,31 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2360796 - 5 units; Placement: area match (High)</t>
+          <t>Site status: Permission Sought; Permission: 24179002 - 18 units on 0.82ha. ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-3</t>
+          <t>CTY-BRUFF-4</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Bruff – site 3</t>
+          <t>Bruff – site 4</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1.377</v>
+        <v>0.234</v>
       </c>
       <c r="E56" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -5827,31 +5827,31 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2560947 - 8 units on  0.349; Placement: area match (High); clipped by consent 2560947</t>
+          <t>Site status: Permission Granted; Permission: 2360796 - 5 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-1</t>
+          <t>CTY-BRUFF-3</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cappamore – site 1</t>
+          <t>Bruff – site 3</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.5620000000000001</v>
+        <v>1.411</v>
       </c>
       <c r="E57" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -5860,31 +5860,31 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 221352 - 17 units; Placement: area match (High); clipped by consent 221352</t>
+          <t>Site status: Permission Granted; Permission: 2560947 - 8 units on  0.349; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-2</t>
+          <t>CTY-CAPPAMORE-1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cappamore – site 2</t>
+          <t>Cappamore – site 1</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.66</v>
+        <v>1.327</v>
       </c>
       <c r="E58" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -5893,31 +5893,31 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Under Construction; Permission: 221352 - 17 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-3</t>
+          <t>CTY-CAPPAMORE-2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Cappamore – site 3</t>
+          <t>Cappamore – site 2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1.012</v>
+        <v>0.66</v>
       </c>
       <c r="E59" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -5926,19 +5926,19 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 23529 - 22 units; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-4</t>
+          <t>CTY-CAPPAMORE-3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Cappamore – site 4</t>
+          <t>Cappamore – site 3</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -5947,10 +5947,10 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.062</v>
+        <v>1.012</v>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -5959,31 +5959,31 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 19872 - 10 units; Placement: area match (High); clipped by consent 19872</t>
+          <t>Site status: Under Construction; Permission: 23529 - 22 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CTY-CROOM-1</t>
+          <t>CTY-CAPPAMORE-4</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Croom – site 1</t>
+          <t>Cappamore – site 4</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Residential Development Area - Phase 1</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.494</v>
+        <v>0.289</v>
       </c>
       <c r="E61" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -5992,31 +5992,31 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Under Construction; Permission: 19872 - 10 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CTY-CROOM-2</t>
+          <t>CTY-CAPPAMORE-5</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Croom – site 2</t>
+          <t>Cappamore – site 5</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Residential Development Area - Phase 1</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>2.951</v>
+        <v>0.18</v>
       </c>
       <c r="E62" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -6025,31 +6025,31 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 21630 - 51 units on 2.007; Reduced site area available due to road construction ; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Permission Granted; Permission: 2260015 - 6 units; 2461101 - 7 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CTY-CROOM-3</t>
+          <t>CTY-CAPPAMORE-6</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Croom – site 3</t>
+          <t>Cappamore – site 6</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites - Phase 1</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.369</v>
+        <v>0.116</v>
       </c>
       <c r="E63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -6058,19 +6058,19 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Site status: Complete; Permission: 21649 - 1 unit, 201219 - 1 unit; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Under Construction; Developing in conjunction with site 1 ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CTY-CROOM-5</t>
+          <t>CTY-CROOM-1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Croom – site 5</t>
+          <t>Croom – site 1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -6079,10 +6079,10 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>4.06</v>
+        <v>0.494</v>
       </c>
       <c r="E64" t="n">
-        <v>89</v>
+        <v>11</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -6098,12 +6098,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CTY-CROOM-6</t>
+          <t>CTY-CROOM-2</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Croom – site 6</t>
+          <t>Croom – site 2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -6112,10 +6112,10 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>2.007</v>
+        <v>2.951</v>
       </c>
       <c r="E65" t="n">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -6124,19 +6124,19 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Site status: Complete; Permission: 22267 - 56 units; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Permission Granted; Permission: 21630 - 51 units on 2.007; Reduced site area available due to road construction ; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CTY-CROOM-7</t>
+          <t>CTY-CROOM-3</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Croom – site 7</t>
+          <t>Croom – site 3</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -6145,10 +6145,10 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>2.677</v>
+        <v>0.369</v>
       </c>
       <c r="E66" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -6157,31 +6157,31 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Complete; Permission: 21649 - 1 unit, 201219 - 1 unit; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-1</t>
+          <t>CTY-CROOM-5</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Hospital – site 1</t>
+          <t>Croom – site 5</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Development Area - Phase 1</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.627</v>
+        <v>4.06</v>
       </c>
       <c r="E67" t="n">
-        <v>14</v>
+        <v>89</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -6190,31 +6190,31 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Pre Planning 16801 - 21 units; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-2</t>
+          <t>CTY-CROOM-6</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Hospital – site 2</t>
+          <t>Croom – site 6</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Development Area - Phase 1</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>1.001</v>
+        <v>2.007</v>
       </c>
       <c r="E68" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -6223,31 +6223,31 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Complete; Permission: 22267 - 56 units; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-3</t>
+          <t>CTY-CROOM-7</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Hospital – site 3</t>
+          <t>Croom – site 7</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites - Phase 1</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.674</v>
+        <v>2.677</v>
       </c>
       <c r="E69" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -6256,31 +6256,31 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-4</t>
+          <t>CTY-CROOM-8</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Hospital – site 4</t>
+          <t>Croom – site 8</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>Residential Development Area - Phase 1</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>1.019</v>
+        <v>0.304</v>
       </c>
       <c r="E70" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -6289,19 +6289,19 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 24151 - 10 units on 0.51ha.; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-1</t>
+          <t>CTY-HOSPITAL-1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Kilfinane – site 1</t>
+          <t>Hospital – site 1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -6310,10 +6310,10 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.091</v>
+        <v>0.627</v>
       </c>
       <c r="E71" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -6322,19 +6322,19 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 218013 - P8 10 units; Under construction; Placement: area match (High); clipped by consent 218013</t>
+          <t>Site status: No Permission Sought; Pre Planning 16801 - 21 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-2</t>
+          <t>CTY-HOSPITAL-2</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Kilfinane – site 2</t>
+          <t>Hospital – site 2</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -6343,10 +6343,10 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.317</v>
+        <v>1.001</v>
       </c>
       <c r="E72" t="n">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -6362,12 +6362,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-3</t>
+          <t>CTY-HOSPITAL-3</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Kilfinane – site 3</t>
+          <t>Hospital – site 3</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -6376,10 +6376,10 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.821</v>
+        <v>0.674</v>
       </c>
       <c r="E73" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -6395,24 +6395,24 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-4</t>
+          <t>CTY-HOSPITAL-4</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Kilfinane – site 4</t>
+          <t>Hospital – site 4</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.713</v>
+        <v>1.019</v>
       </c>
       <c r="E74" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -6421,31 +6421,31 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Site Assembly Required; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-5</t>
+          <t>CTY-KILFINANE-1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Kilfinane – site 5</t>
+          <t>Kilfinane – site 1</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>1.547</v>
+        <v>0.415</v>
       </c>
       <c r="E75" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -6454,19 +6454,19 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Under Construction; Permission: 218013 - P8 10 units; Under construction; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CTY-MURROE-1</t>
+          <t>CTY-KILFINANE-2</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Murroe – site 1</t>
+          <t>Kilfinane – site 2</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -6475,10 +6475,10 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>1.808</v>
+        <v>0.317</v>
       </c>
       <c r="E76" t="n">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -6494,12 +6494,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CTY-MURROE-2</t>
+          <t>CTY-KILFINANE-3</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Murroe – site 2</t>
+          <t>Kilfinane – site 3</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -6508,10 +6508,10 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.997</v>
+        <v>0.821</v>
       </c>
       <c r="E77" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -6527,24 +6527,24 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CTY-MURROE-4</t>
+          <t>CTY-KILFINANE-4</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Murroe – site 4</t>
+          <t>Kilfinane – site 4</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1.938</v>
+        <v>0.713</v>
       </c>
       <c r="E78" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -6553,31 +6553,31 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Site Assembly Required; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-2</t>
+          <t>CTY-KILFINANE-5</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Patrickswell – site 2</t>
+          <t>Kilfinane – site 5</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1.534</v>
+        <v>1.547</v>
       </c>
       <c r="E79" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -6586,31 +6586,31 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High); clipped by consent 18346; clipped by consent 2560156</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-17</t>
+          <t>CTY-MURROE-1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Patrickswell – site 17</t>
+          <t>Murroe – site 1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.4</v>
+        <v>1.808</v>
       </c>
       <c r="E80" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -6619,19 +6619,19 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Site status: No Permission ; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-3</t>
+          <t>CTY-MURROE-2</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Patrickswell – site 3</t>
+          <t>Murroe – site 2</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -6640,10 +6640,10 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.42</v>
+        <v>0.997</v>
       </c>
       <c r="E81" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -6652,19 +6652,19 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2560633 - 6 units  on 0.42; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-8</t>
+          <t>CTY-MURROE-3</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Patrickswell – site 8</t>
+          <t>Murroe – site 3</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -6673,10 +6673,10 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1.772</v>
+        <v>1.082</v>
       </c>
       <c r="E82" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -6685,31 +6685,31 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2360144 - 44 units; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 191298 - 27 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-9</t>
+          <t>CTY-MURROE-4</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Patrickswell – site 9</t>
+          <t>Murroe – site 4</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.39</v>
+        <v>1.938</v>
       </c>
       <c r="E83" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -6718,19 +6718,19 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 19444 - 16 units, 181193 - 48 units; Placement: area match (High); clipped by consent 181193; clipped by consent 19444</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-10</t>
+          <t>CTY-PATRICKSWELL-1</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Patrickswell – site 10</t>
+          <t>Patrickswell – site 1</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -6739,10 +6739,10 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.867</v>
+        <v>4.086</v>
       </c>
       <c r="E84" t="n">
-        <v>19</v>
+        <v>90</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -6751,19 +6751,19 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2560156 - 63 units on 3.040, 2560653 - 40 units on 2.660; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-11</t>
+          <t>CTY-PATRICKSWELL-2</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Patrickswell – site 11</t>
+          <t>Patrickswell – site 2</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -6772,10 +6772,10 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0.386</v>
+        <v>2.935</v>
       </c>
       <c r="E85" t="n">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -6784,289 +6784,325 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Site status: Complete; Permission: 19689 - 8 units; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-U1</t>
+          <t>CTY-PATRICKSWELL-14</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Newcastle West – site U1</t>
+          <t>Patrickswell – site 14</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Town Centre</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>3.815</v>
+        <v>4.773</v>
       </c>
       <c r="E86" t="n">
-        <v>0</v>
-      </c>
-      <c r="F86" t="inlineStr"/>
+        <v>48</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: Commencement Notice but no works; Permission: 20281 - 36, 25/87 - 55 outline; 2561228 - 55 permission consequent new app; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-U2</t>
+          <t>CTY-PATRICKSWELL-17</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Newcastle West – site U2</t>
+          <t>Patrickswell – site 17</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Enterprise and Employment</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>25.055</v>
+        <v>0.4</v>
       </c>
       <c r="E87" t="n">
-        <v>0</v>
-      </c>
-      <c r="F87" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: No Permission ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-U1</t>
+          <t>CTY-PATRICKSWELL-3</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Rathkeale – site U1</t>
+          <t>Patrickswell – site 3</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Enterprise and Employment</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>17.768</v>
+        <v>0.42</v>
       </c>
       <c r="E88" t="n">
-        <v>0</v>
-      </c>
-      <c r="F88" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: Permission Granted; Permission: 2560633 - 6 units  on 0.42; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-U2</t>
+          <t>CTY-PATRICKSWELL-4</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Rathkeale – site U2</t>
+          <t>Patrickswell – site 4</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Enterprise and Employment</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>14.728</v>
+        <v>0.483</v>
       </c>
       <c r="E89" t="n">
-        <v>0</v>
-      </c>
-      <c r="F89" t="inlineStr"/>
+        <v>11</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: Complete; Permission: 21873 - 5 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-U3</t>
+          <t>CTY-PATRICKSWELL-7</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Rathkeale – site U3</t>
+          <t>Patrickswell – site 7</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Enterprise and Employment</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>12.896</v>
+        <v>2.84</v>
       </c>
       <c r="E90" t="n">
-        <v>0</v>
-      </c>
-      <c r="F90" t="inlineStr"/>
+        <v>62</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: Under Construction; Permission: 221318 - 51 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U1</t>
+          <t>CTY-PATRICKSWELL-8</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Askeaton – site U1</t>
+          <t>Patrickswell – site 8</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Resi Service Site Phase 2</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.86</v>
+        <v>1.772</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
-      </c>
-      <c r="F91" t="inlineStr"/>
+        <v>39</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: Permission Granted; Permission: 2360144 - 44 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U2</t>
+          <t>CTY-PATRICKSWELL-9</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Askeaton – site U2</t>
+          <t>Patrickswell – site 9</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Resi Service Site Phase 1</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>1.182</v>
+        <v>2.398</v>
       </c>
       <c r="E92" t="n">
-        <v>0</v>
-      </c>
-      <c r="F92" t="inlineStr"/>
+        <v>53</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: Under Construction; Permission: 19444 - 16 units, 181193 - 48 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U3</t>
+          <t>CTY-PATRICKSWELL-10</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Askeaton – site U3</t>
+          <t>Patrickswell – site 10</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Resi Development Area Phase 1</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>1.04</v>
+        <v>0.867</v>
       </c>
       <c r="E93" t="n">
-        <v>0</v>
-      </c>
-      <c r="F93" t="inlineStr"/>
+        <v>19</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U4</t>
+          <t>CTY-PATRICKSWELL-11</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Askeaton – site U4</t>
+          <t>Patrickswell – site 11</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Resi Development Area Phase 1</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>7.428</v>
+        <v>0.386</v>
       </c>
       <c r="E94" t="n">
-        <v>0</v>
-      </c>
-      <c r="F94" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: Complete; Permission: 19689 - 8 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U5</t>
+          <t>CTY-NEWCASTLEWES-U1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Askeaton – site U5</t>
+          <t>Newcastle West – site U1</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Resi Service Site Phase 2</t>
+          <t>Town Centre</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>2.098</v>
+        <v>3.815</v>
       </c>
       <c r="E95" t="n">
         <v>0</v>
@@ -7081,21 +7117,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U6</t>
+          <t>CTY-NEWCASTLEWES-U2</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Askeaton – site U6</t>
+          <t>Newcastle West – site U2</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Resi Service Site Phase 1</t>
+          <t>Enterprise and Employment</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>2.684</v>
+        <v>25.055</v>
       </c>
       <c r="E96" t="n">
         <v>0</v>
@@ -7110,321 +7146,285 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CTY-BALLINGARRY-1</t>
+          <t>CTY-RATHKEALE-U1</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Ballingarry – site 1</t>
+          <t>Rathkeale – site U1</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Enterprise and Employment</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>1.75</v>
+        <v>17.768</v>
       </c>
       <c r="E97" t="n">
-        <v>38</v>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CTY-BALLINGARRY-2</t>
+          <t>CTY-RATHKEALE-U2</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Ballingarry – site 2</t>
+          <t>Rathkeale – site U2</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>Enterprise and Employment</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>1.057</v>
+        <v>14.728</v>
       </c>
       <c r="E98" t="n">
-        <v>11</v>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CTY-BALLINGARRY-3</t>
+          <t>CTY-RATHKEALE-U3</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Ballingarry – site 3</t>
+          <t>Rathkeale – site U3</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>Enterprise and Employment</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>2.903</v>
+        <v>12.896</v>
       </c>
       <c r="E99" t="n">
-        <v>29</v>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CTY-BRUREE-1</t>
+          <t>CTY-ASKEATON-U1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Bruree – site 1</t>
+          <t>Askeaton – site U1</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Resi Service Site Phase 2</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>1.15</v>
+        <v>0.86</v>
       </c>
       <c r="E100" t="n">
-        <v>25</v>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CTY-BRUREE-2</t>
+          <t>CTY-ASKEATON-U2</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Bruree – site 2</t>
+          <t>Askeaton – site U2</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Resi Service Site Phase 1</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.247</v>
+        <v>1.182</v>
       </c>
       <c r="E101" t="n">
-        <v>5</v>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CTY-BRUREE-3</t>
+          <t>CTY-ASKEATON-U3</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Bruree – site 3</t>
+          <t>Askeaton – site U3</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>Resi Development Area Phase 1</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.736</v>
+        <v>1.04</v>
       </c>
       <c r="E102" t="n">
-        <v>7</v>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CTY-DROMCOLLIHER-1</t>
+          <t>CTY-ASKEATON-U4</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 1</t>
+          <t>Askeaton – site U4</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Resi Development Area Phase 1</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.8080000000000001</v>
+        <v>7.428</v>
       </c>
       <c r="E103" t="n">
-        <v>18</v>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CTY-DROMCOLLIHER-2</t>
+          <t>CTY-ASKEATON-U5</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 2</t>
+          <t>Askeaton – site U5</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Resi Service Site Phase 2</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.07099999999999999</v>
+        <v>2.098</v>
       </c>
       <c r="E104" t="n">
-        <v>2</v>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CTY-DROMCOLLIHER-3</t>
+          <t>CTY-ASKEATON-U6</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 3</t>
+          <t>Askeaton – site U6</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Resi Service Site Phase 1</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.845</v>
+        <v>2.684</v>
       </c>
       <c r="E105" t="n">
-        <v>19</v>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CTY-DROMCOLLIHER-4</t>
+          <t>CTY-BALLINGARRY-1</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 4</t>
+          <t>Ballingarry – site 1</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Residential</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.773</v>
+        <v>1.75</v>
       </c>
       <c r="E106" t="n">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -7440,24 +7440,24 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CTY-FOYNES-1</t>
+          <t>CTY-BALLINGARRY-2</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Foynes – site 1</t>
+          <t>Ballingarry – site 2</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>3.497</v>
+        <v>1.057</v>
       </c>
       <c r="E107" t="n">
-        <v>56</v>
+        <v>11</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -7473,24 +7473,24 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CTY-GLIN-1</t>
+          <t>CTY-BALLINGARRY-3</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Glin – site 1</t>
+          <t>Ballingarry – site 3</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Mixed Use</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>1.613</v>
+        <v>2.903</v>
       </c>
       <c r="E108" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -7506,12 +7506,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>CTY-GLIN-2</t>
+          <t>CTY-BRUREE-1</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Glin – site 2</t>
+          <t>Bruree – site 1</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -7520,10 +7520,10 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.527</v>
+        <v>1.15</v>
       </c>
       <c r="E109" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -7539,24 +7539,24 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>CTY-GLIN-3</t>
+          <t>CTY-BRUREE-2</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Glin – site 3</t>
+          <t>Bruree – site 2</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Residential</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.965</v>
+        <v>0.247</v>
       </c>
       <c r="E110" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -7572,24 +7572,24 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CTY-GLIN-4</t>
+          <t>CTY-BRUREE-3</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Glin – site 4</t>
+          <t>Bruree – site 3</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>1.25</v>
+        <v>0.736</v>
       </c>
       <c r="E111" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
@@ -7605,28 +7605,28 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-5</t>
+          <t>CTY-DROMCOLLIHER-1</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Hospital – site 5</t>
+          <t>Dromcolliher – site 1</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Enterprise &amp; Employment</t>
+          <t>New Residential</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>2.675</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="E112" t="n">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Estimate (council audit recorded no capacity): developable area x density</t>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -7638,12 +7638,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CTY-PALLASGREEN-2</t>
+          <t>CTY-DROMCOLLIHER-2</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Pallasgreen – site 2</t>
+          <t>Dromcolliher – site 2</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -7652,10 +7652,10 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>1.424</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="E113" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -7671,12 +7671,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CTY-PALLASGREEN-1</t>
+          <t>CTY-DROMCOLLIHER-3</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Pallasgreen – site 1</t>
+          <t>Dromcolliher – site 3</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -7685,10 +7685,10 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.613</v>
+        <v>0.845</v>
       </c>
       <c r="E114" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
@@ -7704,12 +7704,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CTY-PALLASGREEN-3</t>
+          <t>CTY-DROMCOLLIHER-4</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Pallasgreen – site 3</t>
+          <t>Dromcolliher – site 4</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -7718,10 +7718,10 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>1.07</v>
+        <v>0.773</v>
       </c>
       <c r="E115" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
@@ -7737,24 +7737,24 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CTY-PALLASKENRY-4</t>
+          <t>CTY-FOYNES-1</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Pallaskenry – site 4</t>
+          <t>Foynes – site 1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Residential</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0.271</v>
+        <v>3.497</v>
       </c>
       <c r="E116" t="n">
-        <v>3</v>
+        <v>56</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -7763,38 +7763,335 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon; clipped by consent 24352</t>
+          <t>Placement: 2022 polygon</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
+          <t>CTY-GLIN-1</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Glin – site 1</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Mixed Use</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>1.613</v>
+      </c>
+      <c r="E117" t="n">
+        <v>36</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>CTY-GLIN-2</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Glin – site 2</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>0.527</v>
+      </c>
+      <c r="E118" t="n">
+        <v>12</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>CTY-GLIN-3</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Glin – site 3</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="E119" t="n">
+        <v>10</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>CTY-GLIN-4</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Glin – site 4</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E120" t="n">
+        <v>27</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>CTY-HOSPITAL-5</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Hospital – site 5</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Enterprise &amp; Employment</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>2.675</v>
+      </c>
+      <c r="E121" t="n">
+        <v>67</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Estimate (council audit recorded no capacity): developable area x density</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>CTY-PALLASGREEN-2</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Pallasgreen – site 2</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>1.424</v>
+      </c>
+      <c r="E122" t="n">
+        <v>31</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>CTY-PALLASGREEN-1</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Pallasgreen – site 1</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>0.613</v>
+      </c>
+      <c r="E123" t="n">
+        <v>14</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>CTY-PALLASGREEN-3</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Pallasgreen – site 3</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E124" t="n">
+        <v>11</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>CTY-PALLASKENRY-4</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Pallaskenry – site 4</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="E125" t="n">
+        <v>3</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon; clipped by consent 24352</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
           <t>CTY-PALLASKENRY-3</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B126" t="inlineStr">
         <is>
           <t>Pallaskenry – site 3</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C126" t="inlineStr">
         <is>
           <t>New Residential</t>
         </is>
       </c>
-      <c r="D117" t="n">
+      <c r="D126" t="n">
         <v>0.753</v>
       </c>
-      <c r="E117" t="n">
+      <c r="E126" t="n">
         <v>17</v>
       </c>
-      <c r="F117" t="inlineStr">
+      <c r="F126" t="inlineStr">
         <is>
           <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
+      <c r="G126" t="inlineStr">
         <is>
           <t>Placement: 2022 polygon</t>
         </is>
@@ -8044,7 +8341,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PC-181193</t>
+          <t>CTY-PATRICKSWELL-9</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8456,7 +8753,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PC-21594</t>
+          <t>CTY-ABBEYFEALE-5</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -9172,7 +9469,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PC-2560156</t>
+          <t>CTY-PATRICKSWELL-1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -9292,7 +9589,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PC-2561228</t>
+          <t>CTY-PATRICKSWELL-14</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -9828,7 +10125,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PC-24151</t>
+          <t>CTY-CROOM-8</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -10154,7 +10451,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.238</v>
+        <v>1.5</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -10179,7 +10476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10455,18 +10752,180 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>CTY-NEWCASTLEWES-6</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Newcastle West – site 6</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CTY-CAPPAMORE-4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Cappamore – site 4</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CTY-CAPPAMORE-5</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Cappamore – site 5</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CTY-CROOM-8</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Croom – site 8</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>7</v>
+      </c>
+      <c r="D19" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CTY-KILFINANE-1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Kilfinane – site 1</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>9</v>
+      </c>
+      <c r="D20" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CTY-MURROE-3</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Murroe – site 3</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>24</v>
+      </c>
+      <c r="D21" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 1</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>90</v>
+      </c>
+      <c r="D22" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-14</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 14</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>48</v>
+      </c>
+      <c r="D23" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CTY-PATRICKSWELL-9</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Patrickswell – site 9</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>53</v>
+      </c>
+      <c r="D24" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>CTY-PATRICKSWELL-11</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Patrickswell – site 11</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C25" t="n">
         <v>8</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D25" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: include every council-supplied polygon; town-average density where no council capacity
- hand-drawn Newcastle West sites (6 polygons) loaded; polygons without a plan name no longer dropped
- capacity for unmatched council sites = area x town average density by site type from the council Excel

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-26 15:12</t>
+          <t>2026-10-26 15:46</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>448 parcels</t>
+          <t>452 parcels</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{'Inside catchment': 361, 'Rest of county': 46, 'Edge of settlement (within 500 m)': 31, 'Zoned in': 9, 'Named in scheme, within 2 km': 1}</t>
+          <t>{'Inside catchment': 364, 'Rest of county': 46, 'Edge of settlement (within 500 m)': 32, 'Zoned in': 9, 'Named in scheme, within 2 km': 1}</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>125 county audit parcels, 3,486 homes</t>
+          <t>129 county audit parcels, 6,257 homes</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -4000,7 +4000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4076,45 +4076,45 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-5</t>
+          <t>CTY-NEWCASTLEWES-3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Newcastle West – site 5</t>
+          <t>Newcastle West – site 3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Town Centre</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>12.5</v>
+        <v>1.2</v>
       </c>
       <c r="E3" t="n">
-        <v>438</v>
+        <v>40</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Site status: Partially Development - Reduced Area Available; Permission: 22840 - 93 units; Is part of this built out?; Placement: area match (High)</t>
+          <t>Site status: No Permission; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-6</t>
+          <t>CTY-NEWCASTLEWES-5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Newcastle West – site 6</t>
+          <t>Newcastle West – site 5</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4123,31 +4123,31 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.5</v>
+        <v>12.5</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>438</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Site status: Partially Development - Reduced Area Available; Permission: 2360706 - 53 units, 17383 - 54 units; Placement: area match (High)</t>
+          <t>Site status: Partially Development - Reduced Area Available; Permission: 22840 - 93 units; Is part of this built out?; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-8</t>
+          <t>CTY-NEWCASTLEWES-6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Newcastle West – site 8</t>
+          <t>Newcastle West – site 6</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4156,31 +4156,31 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.4</v>
+        <v>1.5</v>
       </c>
       <c r="E5" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Site status: Permission Sought; Permission: 2660575 - 30 units, 0.428ha. - FI; Placement: area match (High)</t>
+          <t>Site status: Partially Development - Reduced Area Available; Permission: 2360706 - 53 units, 17383 - 54 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-11D</t>
+          <t>CTY-NEWCASTLEWES-8</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Newcastle West – site 11D</t>
+          <t>Newcastle West – site 8</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4189,31 +4189,31 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.38</v>
+        <v>0.4</v>
       </c>
       <c r="E6" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (High)</t>
+          <t>Site status: Permission Sought; Permission: 2660575 - 30 units, 0.428ha. - FI; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-12</t>
+          <t>CTY-NEWCASTLEWES-11D</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Newcastle West – site 12</t>
+          <t>Newcastle West – site 11D</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4222,14 +4222,14 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.8</v>
+        <v>1.38</v>
       </c>
       <c r="E7" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4241,12 +4241,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-13</t>
+          <t>CTY-NEWCASTLEWES-12</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Newcastle West – site 13</t>
+          <t>Newcastle West – site 12</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4255,31 +4255,31 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.1</v>
+        <v>0.8</v>
       </c>
       <c r="E8" t="n">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2360826 - 14 units; Placement: area match (High)</t>
+          <t>Site status: No Permission; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-14</t>
+          <t>CTY-NEWCASTLEWES-13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Newcastle West – site 14</t>
+          <t>Newcastle West – site 13</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4288,31 +4288,31 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.3</v>
+        <v>2.1</v>
       </c>
       <c r="E9" t="n">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 228020 - P8 21 units; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2360826 - 14 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-17</t>
+          <t>CTY-NEWCASTLEWES-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Newcastle West – site 17</t>
+          <t>Newcastle West – site 14</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4321,64 +4321,64 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1.12</v>
+        <v>1.3</v>
       </c>
       <c r="E10" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Is this land directly accessible to services?; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 228020 - P8 21 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-1</t>
+          <t>CTY-NEWCASTLEWES-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 1</t>
+          <t>Newcastle West – site 17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Town Centre</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.57</v>
+        <v>1.12</v>
       </c>
       <c r="E11" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Requires Site Assembly ; Placement: area match (High)</t>
+          <t>Site status: No Permission; Is this land directly accessible to services?; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-3</t>
+          <t>CTY-ABBEYFEALE-1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 3</t>
+          <t>Abbeyfeale – site 1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4387,14 +4387,14 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.26</v>
+        <v>0.57</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4406,94 +4406,94 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-5</t>
+          <t>CTY-ABBEYFEALE-3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 5</t>
+          <t>Abbeyfeale – site 3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Town Centre</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>4.2</v>
+        <v>0.26</v>
       </c>
       <c r="E13" t="n">
-        <v>92</v>
+        <v>9</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2660232 - 48 unitss, 2.081; 21594 - 68 units, 2.79ha.; 2460606 - 40 units, 1.76ha. Appeal Refused by ACP ; Placement: area match (High)</t>
+          <t>Site status: No Permission; Requires Site Assembly ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-7</t>
+          <t>CTY-ABBEYFEALE-5</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 7</t>
+          <t>Abbeyfeale – site 5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>92</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2660232 - 48 unitss, 2.081; 21594 - 68 units, 2.79ha.; 2460606 - 40 units, 1.76ha. Appeal Refused by ACP ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-8</t>
+          <t>CTY-ABBEYFEALE-7</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 8</t>
+          <t>Abbeyfeale – site 7</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4505,28 +4505,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-9</t>
+          <t>CTY-ABBEYFEALE-8</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 9</t>
+          <t>Abbeyfeale – site 8</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E16" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4538,12 +4538,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CTY-ABBEYFEALE-10</t>
+          <t>CTY-ABBEYFEALE-9</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 10</t>
+          <t>Abbeyfeale – site 9</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -4552,14 +4552,14 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4571,45 +4571,45 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-1</t>
+          <t>CTY-ABBEYFEALE-10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Castleconnell – site 1</t>
+          <t>Abbeyfeale – site 10</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.26</v>
+        <v>0.5</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-2</t>
+          <t>CTY-CASTLECONNEL-1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Castleconnell – site 2</t>
+          <t>Castleconnell – site 1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4618,14 +4618,14 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.63</v>
+        <v>0.26</v>
       </c>
       <c r="E19" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -4637,12 +4637,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-3</t>
+          <t>CTY-CASTLECONNEL-2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Castleconnell – site 3</t>
+          <t>Castleconnell – site 2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4651,14 +4651,14 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="E20" t="n">
         <v>14</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -4670,12 +4670,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-4</t>
+          <t>CTY-CASTLECONNEL-3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Castleconnell – site 4</t>
+          <t>Castleconnell – site 3</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4684,31 +4684,31 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6.1</v>
+        <v>0.62</v>
       </c>
       <c r="E21" t="n">
-        <v>134</v>
+        <v>14</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Site status: Commenced -Reduced area available; Permission: 2360866 - 74 units; Placement: area match (Low), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-5</t>
+          <t>CTY-CASTLECONNEL-4</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Castleconnell – site 5</t>
+          <t>Castleconnell – site 4</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4717,64 +4717,64 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.49</v>
+        <v>6.1</v>
       </c>
       <c r="E22" t="n">
-        <v>11</v>
+        <v>134</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 25327 - 2units; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: Commenced -Reduced area available; Permission: 2360866 - 74 units; Placement: area match (Low), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-6</t>
+          <t>CTY-CASTLECONNEL-5</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Castleconnell – site 6</t>
+          <t>Castleconnell – site 5</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1.1</v>
+        <v>0.49</v>
       </c>
       <c r="E23" t="n">
         <v>11</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Pre Planning 562893 - 25 units; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Permission Granted; Permission: 25327 - 2units; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-8</t>
+          <t>CTY-CASTLECONNEL-6</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Castleconnell – site 8</t>
+          <t>Castleconnell – site 6</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4783,114 +4783,122 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="E24" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: No Permission; Pre Planning 562893 - 25 units; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-9</t>
+          <t>CTY-CASTLECONNEL-8</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Castleconnell – site 9</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
+          <t>Castleconnell – site 8</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
       <c r="D25" t="n">
-        <v>4.009</v>
+        <v>1.6</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
+        <v>16</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; on the council map but not in the Excel; 9/10 order to confirm</t>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CTY-CASTLECONNEL-10</t>
+          <t>CTY-CASTLECONNEL-9</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Castleconnell – site 10</t>
+          <t>Castleconnell – site 9</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="n">
-        <v>6.742</v>
+        <v>4.009</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
+        <v>88</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Area x town average density for resi sites in the council audit (22/ha)</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; on the council map but not in the Excel; 9/10 order to confirm</t>
+          <t>On the council map, not in the Excel: site number and figures to confirm; Placement: council outline; on the council map but not in the Excel; 9/10 order to confirm</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-1</t>
+          <t>CTY-CASTLECONNEL-10</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Caherconlish – site 1</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>New Resi</t>
-        </is>
-      </c>
+          <t>Castleconnell – site 10</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="n">
-        <v>3.58</v>
+        <v>6.742</v>
       </c>
       <c r="E27" t="n">
-        <v>79</v>
+        <v>148</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Area x town average density for resi sites in the council audit (22/ha)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Pre Planning 1032260 - 58 units; Placement: area match (High), confirmed by analyst</t>
+          <t>On the council map, not in the Excel: site number and figures to confirm; Placement: council outline; on the council map but not in the Excel; 9/10 order to confirm</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-2</t>
+          <t>CTY-CAHERCONLISH-1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Caherconlish – site 2</t>
+          <t>Caherconlish – site 1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4899,31 +4907,31 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.439</v>
+        <v>3.58</v>
       </c>
       <c r="E28" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: placed per analyst (council map): west of site 3; two zoning polygons together = 0.44 ha</t>
+          <t>Site status: No Permission; Pre Planning 1032260 - 58 units; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-3</t>
+          <t>CTY-CAHERCONLISH-2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Caherconlish – site 3</t>
+          <t>Caherconlish – site 2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -4932,122 +4940,126 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.234</v>
+        <v>0.439</v>
       </c>
       <c r="E29" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match; confirm (analyst marked the first placement of 3 wrong)</t>
+          <t>Site status: No Permission; Placement: placed per analyst (council map): west of site 3; two zoning polygons together = 0.44 ha</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-5</t>
+          <t>CTY-CAHERCONLISH-3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Caherconlish – site 5</t>
+          <t>Caherconlish – site 3</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>2.085</v>
+        <v>0.234</v>
       </c>
       <c r="E30" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Pre Planning - 1049863 - 110 units; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: area match; confirm (analyst marked the first placement of 3 wrong)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CTY-CAHERCONLISH-7</t>
+          <t>CTY-CAHERCONLISH-5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Caherconlish – site 7</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+          <t>Caherconlish – site 5</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
       <c r="D31" t="n">
-        <v>5.889</v>
+        <v>2.085</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>On the council map, not in the Excel: fill in area, density and capacity; Placement: council outline; site 7 is on the council map but not in the Excel</t>
+          <t>Site status: No Permission; Pre Planning - 1049863 - 110 units; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-1</t>
+          <t>CTY-CAHERCONLISH-7</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Rathkeale – site 1</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>New Resi</t>
-        </is>
-      </c>
+          <t>Caherconlish – site 7</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="n">
-        <v>0.4</v>
+        <v>5.889</v>
       </c>
       <c r="E32" t="n">
-        <v>9</v>
+        <v>130</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Area x town average density for resi sites in the council audit (22/ha)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: placed per analyst (council map): northwest of site 2</t>
+          <t>On the council map, not in the Excel: site number and figures to confirm; Placement: council outline; site 7 is on the council map but not in the Excel</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-2</t>
+          <t>CTY-RATHKEALE-1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Rathkeale – site 2</t>
+          <t>Rathkeale – site 1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5056,31 +5068,31 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1.039</v>
+        <v>0.4</v>
       </c>
       <c r="E33" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: placed per analyst (council map): northwest of site 2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-3</t>
+          <t>CTY-RATHKEALE-2</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Rathkeale – site 3</t>
+          <t>Rathkeale – site 2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5089,14 +5101,14 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1.57</v>
+        <v>1.039</v>
       </c>
       <c r="E34" t="n">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -5108,12 +5120,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-4</t>
+          <t>CTY-RATHKEALE-3</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Rathkeale – site 4</t>
+          <t>Rathkeale – site 3</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5122,14 +5134,14 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.36</v>
+        <v>1.57</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -5141,12 +5153,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-5</t>
+          <t>CTY-RATHKEALE-4</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Rathkeale – site 5</t>
+          <t>Rathkeale – site 4</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5155,14 +5167,14 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.601</v>
+        <v>0.36</v>
       </c>
       <c r="E36" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -5174,12 +5186,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-6</t>
+          <t>CTY-RATHKEALE-5</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Rathkeale – site 6</t>
+          <t>Rathkeale – site 5</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5188,31 +5200,31 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.82</v>
+        <v>0.601</v>
       </c>
       <c r="E37" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: placed per analyst (council map); Excel area 0.82 ha vs polygon 0.38 ha</t>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-7</t>
+          <t>CTY-RATHKEALE-6</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Rathkeale – site 7</t>
+          <t>Rathkeale – site 6</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5221,31 +5233,31 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.27</v>
+        <v>0.82</v>
       </c>
       <c r="E38" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: placed per analyst (council map); Excel area 0.82 ha vs polygon 0.38 ha</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-8</t>
+          <t>CTY-RATHKEALE-7</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Rathkeale – site 8</t>
+          <t>Rathkeale – site 7</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -5254,14 +5266,14 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1.35</v>
+        <v>1.27</v>
       </c>
       <c r="E39" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -5273,28 +5285,28 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-9</t>
+          <t>CTY-RATHKEALE-8</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Rathkeale – site 9</t>
+          <t>Rathkeale – site 8</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.427</v>
+        <v>1.35</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -5306,12 +5318,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-10</t>
+          <t>CTY-RATHKEALE-9</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Rathkeale – site 10</t>
+          <t>Rathkeale – site 9</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -5320,14 +5332,14 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1.785</v>
+        <v>0.427</v>
       </c>
       <c r="E41" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -5339,78 +5351,78 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-1</t>
+          <t>CTY-RATHKEALE-10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Kilmallock – site 1</t>
+          <t>Rathkeale – site 10</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Residential Development Area</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3.88</v>
+        <v>1.785</v>
       </c>
       <c r="E42" t="n">
-        <v>85</v>
+        <v>18</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 2326 - 28 units; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-2</t>
+          <t>CTY-KILMALLOCK-1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Kilmallock – site 2</t>
+          <t>Kilmallock – site 1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>Residential Development Area</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3.79</v>
+        <v>3.88</v>
       </c>
       <c r="E43" t="n">
-        <v>38</v>
+        <v>85</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Pre Planning for 26 units; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: Under Construction; Permission: 2326 - 28 units; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-8</t>
+          <t>CTY-KILMALLOCK-2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Kilmallock – site 8</t>
+          <t>Kilmallock – site 2</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5419,64 +5431,64 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3.73</v>
+        <v>3.79</v>
       </c>
       <c r="E44" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
+          <t>Site status: No Permission; Pre Planning for 26 units; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-9</t>
+          <t>CTY-KILMALLOCK-8</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Kilmallock – site 9</t>
+          <t>Kilmallock – site 8</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Residential Development Area</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>5.33</v>
+        <v>3.73</v>
       </c>
       <c r="E45" t="n">
-        <v>117</v>
+        <v>37</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Site status: No Permission; Placement: area match (Low), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: area match (Medium), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CTY-KILMALLOCK-10</t>
+          <t>CTY-KILMALLOCK-9</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Kilmallock – site 10</t>
+          <t>Kilmallock – site 9</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -5485,64 +5497,64 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4.24</v>
+        <v>5.33</v>
       </c>
       <c r="E46" t="n">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 2460788 - 42 units on 1.64; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission; Placement: area match (Low), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CTY-ADARE-1A</t>
+          <t>CTY-KILMALLOCK-10</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Adare – site 1a</t>
+          <t>Kilmallock – site 10</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Development Area</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1.1</v>
+        <v>4.24</v>
       </c>
       <c r="E47" t="n">
-        <v>24</v>
+        <v>93</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 198010 - P8 31 units &amp; 8 plots; Placement: area match (High)</t>
+          <t>Site status: Under Construction; Permission: 2460788 - 42 units on 1.64; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CTY-ADARE-5</t>
+          <t>CTY-ADARE-1A</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Adare – site 5</t>
+          <t>Adare – site 1a</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5551,31 +5563,31 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="E48" t="n">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 198010 - P8 31 units &amp; 8 plots; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CTY-ADARE-6</t>
+          <t>CTY-ADARE-5</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Adare – site 6</t>
+          <t>Adare – site 5</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5584,14 +5596,14 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.338</v>
+        <v>1.7</v>
       </c>
       <c r="E49" t="n">
-        <v>7</v>
+        <v>37</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -5603,28 +5615,28 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CTY-ADARE-8</t>
+          <t>CTY-ADARE-6</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Adare – site 8</t>
+          <t>Adare – site 6</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.15</v>
+        <v>0.338</v>
       </c>
       <c r="E50" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -5636,28 +5648,28 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-6</t>
+          <t>CTY-ADARE-8</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Askeaton – site 6</t>
+          <t>Adare – site 8</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites - Phase 1</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1.018</v>
+        <v>1.15</v>
       </c>
       <c r="E51" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5669,28 +5681,28 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-10</t>
+          <t>CTY-ASKEATON-6</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Askeaton – site 10</t>
+          <t>Askeaton – site 6</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Residential Development Area - Phase 2</t>
+          <t>Residential Serviced Sites - Phase 1</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>4.719</v>
+        <v>1.018</v>
       </c>
       <c r="E52" t="n">
-        <v>104</v>
+        <v>10</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -5702,28 +5714,28 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-9</t>
+          <t>CTY-ASKEATON-10</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Askeaton – site 9</t>
+          <t>Askeaton – site 10</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites - Phase 2</t>
+          <t>Residential Development Area - Phase 2</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2.459</v>
+        <v>4.719</v>
       </c>
       <c r="E53" t="n">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -5735,45 +5747,45 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-1</t>
+          <t>CTY-ASKEATON-9</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Bruff – site 1</t>
+          <t>Askeaton – site 9</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites - Phase 2</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>3.277</v>
+        <v>2.459</v>
       </c>
       <c r="E54" t="n">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2360794 - 74 units; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-2</t>
+          <t>CTY-BRUFF-1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Bruff – site 2</t>
+          <t>Bruff – site 1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -5782,31 +5794,31 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.679</v>
+        <v>3.277</v>
       </c>
       <c r="E55" t="n">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Site status: Permission Sought; Permission: 24179002 - 18 units on 0.82ha. ; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2360794 - 74 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-4</t>
+          <t>CTY-BRUFF-2</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Bruff – site 4</t>
+          <t>Bruff – site 2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -5815,163 +5827,163 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.234</v>
+        <v>0.679</v>
       </c>
       <c r="E56" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2360796 - 5 units; Placement: area match (High)</t>
+          <t>Site status: Permission Sought; Permission: 24179002 - 18 units on 0.82ha. ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CTY-BRUFF-3</t>
+          <t>CTY-BRUFF-4</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Bruff – site 3</t>
+          <t>Bruff – site 4</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1.411</v>
+        <v>0.234</v>
       </c>
       <c r="E57" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2560947 - 8 units on  0.349; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2360796 - 5 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-1</t>
+          <t>CTY-BRUFF-3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cappamore – site 1</t>
+          <t>Bruff – site 3</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1.327</v>
+        <v>1.411</v>
       </c>
       <c r="E58" t="n">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 221352 - 17 units; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2560947 - 8 units on  0.349; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-2</t>
+          <t>CTY-CAPPAMORE-1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Cappamore – site 2</t>
+          <t>Cappamore – site 1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.66</v>
+        <v>1.327</v>
       </c>
       <c r="E59" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Under Construction; Permission: 221352 - 17 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-3</t>
+          <t>CTY-CAPPAMORE-2</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Cappamore – site 3</t>
+          <t>Cappamore – site 2</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1.012</v>
+        <v>0.66</v>
       </c>
       <c r="E60" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 23529 - 22 units; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-4</t>
+          <t>CTY-CAPPAMORE-3</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Cappamore – site 4</t>
+          <t>Cappamore – site 3</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -5980,31 +5992,31 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.289</v>
+        <v>1.012</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 19872 - 10 units; Placement: area match (High)</t>
+          <t>Site status: Under Construction; Permission: 23529 - 22 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-5</t>
+          <t>CTY-CAPPAMORE-4</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Cappamore – site 5</t>
+          <t>Cappamore – site 4</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -6013,31 +6025,31 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.18</v>
+        <v>0.289</v>
       </c>
       <c r="E62" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2260015 - 6 units; 2461101 - 7 units; Placement: area match (High)</t>
+          <t>Site status: Under Construction; Permission: 19872 - 10 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CTY-CAPPAMORE-6</t>
+          <t>CTY-CAPPAMORE-5</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Cappamore – site 6</t>
+          <t>Cappamore – site 5</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -6046,64 +6058,64 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.116</v>
+        <v>0.18</v>
       </c>
       <c r="E63" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Developing in conjunction with site 1 ; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2260015 - 6 units; 2461101 - 7 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CTY-CROOM-1</t>
+          <t>CTY-CAPPAMORE-6</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Croom – site 1</t>
+          <t>Cappamore – site 6</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Residential Development Area - Phase 1</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.494</v>
+        <v>0.116</v>
       </c>
       <c r="E64" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Under Construction; Developing in conjunction with site 1 ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CTY-CROOM-2</t>
+          <t>CTY-CROOM-1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Croom – site 2</t>
+          <t>Croom – site 1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -6112,97 +6124,97 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>2.951</v>
+        <v>0.494</v>
       </c>
       <c r="E65" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 21630 - 51 units on 2.007; Reduced site area available due to road construction ; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CTY-CROOM-3</t>
+          <t>CTY-CROOM-2</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Croom – site 3</t>
+          <t>Croom – site 2</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites - Phase 1</t>
+          <t>Residential Development Area - Phase 1</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.369</v>
+        <v>2.951</v>
       </c>
       <c r="E66" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Site status: Complete; Permission: 21649 - 1 unit, 201219 - 1 unit; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Permission Granted; Permission: 21630 - 51 units on 2.007; Reduced site area available due to road construction ; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CTY-CROOM-5</t>
+          <t>CTY-CROOM-3</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Croom – site 5</t>
+          <t>Croom – site 3</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Residential Development Area - Phase 1</t>
+          <t>Residential Serviced Sites - Phase 1</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>4.06</v>
+        <v>0.369</v>
       </c>
       <c r="E67" t="n">
-        <v>89</v>
+        <v>4</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Complete; Permission: 21649 - 1 unit, 201219 - 1 unit; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CTY-CROOM-6</t>
+          <t>CTY-CROOM-5</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Croom – site 6</t>
+          <t>Croom – site 5</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -6211,130 +6223,130 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>2.007</v>
+        <v>4.06</v>
       </c>
       <c r="E68" t="n">
-        <v>44</v>
+        <v>89</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Site status: Complete; Permission: 22267 - 56 units; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CTY-CROOM-7</t>
+          <t>CTY-CROOM-6</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Croom – site 7</t>
+          <t>Croom – site 6</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites - Phase 1</t>
+          <t>Residential Development Area - Phase 1</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>2.677</v>
+        <v>2.007</v>
       </c>
       <c r="E69" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: Complete; Permission: 22267 - 56 units; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CTY-CROOM-8</t>
+          <t>CTY-CROOM-7</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Croom – site 8</t>
+          <t>Croom – site 7</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Residential Development Area - Phase 1</t>
+          <t>Residential Serviced Sites - Phase 1</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.304</v>
+        <v>2.677</v>
       </c>
       <c r="E70" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 24151 - 10 units on 0.51ha.; Placement: area match (High), confirmed by analyst</t>
+          <t>Site status: No Permission Sought; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-1</t>
+          <t>CTY-CROOM-8</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Hospital – site 1</t>
+          <t>Croom – site 8</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Development Area - Phase 1</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.627</v>
+        <v>0.304</v>
       </c>
       <c r="E71" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Pre Planning 16801 - 21 units; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 24151 - 10 units on 0.51ha.; Placement: area match (High), confirmed by analyst</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-2</t>
+          <t>CTY-HOSPITAL-1</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Hospital – site 2</t>
+          <t>Hospital – site 1</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -6343,31 +6355,31 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>1.001</v>
+        <v>0.627</v>
       </c>
       <c r="E72" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Pre Planning 16801 - 21 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-3</t>
+          <t>CTY-HOSPITAL-2</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Hospital – site 3</t>
+          <t>Hospital – site 2</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -6376,14 +6388,14 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.674</v>
+        <v>1.001</v>
       </c>
       <c r="E73" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -6395,28 +6407,28 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-4</t>
+          <t>CTY-HOSPITAL-3</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Hospital – site 4</t>
+          <t>Hospital – site 3</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>1.019</v>
+        <v>0.674</v>
       </c>
       <c r="E74" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -6428,45 +6440,45 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-1</t>
+          <t>CTY-HOSPITAL-4</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Kilfinane – site 1</t>
+          <t>Hospital – site 4</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.415</v>
+        <v>1.019</v>
       </c>
       <c r="E75" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 218013 - P8 10 units; Under construction; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-2</t>
+          <t>CTY-KILFINANE-1</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Kilfinane – site 2</t>
+          <t>Kilfinane – site 1</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -6475,31 +6487,31 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.317</v>
+        <v>0.415</v>
       </c>
       <c r="E76" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Under Construction; Permission: 218013 - P8 10 units; Under construction; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-3</t>
+          <t>CTY-KILFINANE-2</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Kilfinane – site 3</t>
+          <t>Kilfinane – site 2</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -6508,14 +6520,14 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.821</v>
+        <v>0.317</v>
       </c>
       <c r="E77" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -6527,12 +6539,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-4</t>
+          <t>CTY-KILFINANE-3</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Kilfinane – site 4</t>
+          <t>Kilfinane – site 3</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -6541,80 +6553,80 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.713</v>
+        <v>0.821</v>
       </c>
       <c r="E78" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Site Assembly Required; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CTY-KILFINANE-5</t>
+          <t>CTY-KILFINANE-4</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Kilfinane – site 5</t>
+          <t>Kilfinane – site 4</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1.547</v>
+        <v>0.713</v>
       </c>
       <c r="E79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Site Assembly Required; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CTY-MURROE-1</t>
+          <t>CTY-KILFINANE-5</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Murroe – site 1</t>
+          <t>Kilfinane – site 5</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>1.808</v>
+        <v>1.547</v>
       </c>
       <c r="E80" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -6626,12 +6638,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CTY-MURROE-2</t>
+          <t>CTY-MURROE-1</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Murroe – site 2</t>
+          <t>Murroe – site 1</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -6640,14 +6652,14 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.997</v>
+        <v>1.808</v>
       </c>
       <c r="E81" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -6659,12 +6671,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CTY-MURROE-3</t>
+          <t>CTY-MURROE-2</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Murroe – site 3</t>
+          <t>Murroe – site 2</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -6673,97 +6685,97 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1.082</v>
+        <v>0.997</v>
       </c>
       <c r="E82" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 191298 - 27 units; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CTY-MURROE-4</t>
+          <t>CTY-MURROE-3</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Murroe – site 4</t>
+          <t>Murroe – site 3</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1.938</v>
+        <v>1.082</v>
       </c>
       <c r="E83" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 191298 - 27 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-1</t>
+          <t>CTY-MURROE-4</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Patrickswell – site 1</t>
+          <t>Murroe – site 4</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>4.086</v>
+        <v>1.938</v>
       </c>
       <c r="E84" t="n">
-        <v>90</v>
+        <v>19</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2560156 - 63 units on 3.040, 2560653 - 40 units on 2.660; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-2</t>
+          <t>CTY-PATRICKSWELL-1</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Patrickswell – site 2</t>
+          <t>Patrickswell – site 1</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -6772,64 +6784,64 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>2.935</v>
+        <v>4.086</v>
       </c>
       <c r="E85" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2560156 - 63 units on 3.040, 2560653 - 40 units on 2.660; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-14</t>
+          <t>CTY-PATRICKSWELL-2</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Patrickswell – site 14</t>
+          <t>Patrickswell – site 2</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>4.773</v>
+        <v>2.935</v>
       </c>
       <c r="E86" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Site status: Commencement Notice but no works; Permission: 20281 - 36, 25/87 - 55 outline; 2561228 - 55 permission consequent new app; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-17</t>
+          <t>CTY-PATRICKSWELL-14</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Patrickswell – site 17</t>
+          <t>Patrickswell – site 14</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -6838,64 +6850,64 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.4</v>
+        <v>4.773</v>
       </c>
       <c r="E87" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Site status: No Permission ; Placement: area match (High)</t>
+          <t>Site status: Commencement Notice but no works; Permission: 20281 - 36, 25/87 - 55 outline; 2561228 - 55 permission consequent new app; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-3</t>
+          <t>CTY-PATRICKSWELL-17</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Patrickswell – site 3</t>
+          <t>Patrickswell – site 17</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>New Resi</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="E88" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2560633 - 6 units  on 0.42; Placement: area match (High)</t>
+          <t>Site status: No Permission ; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-4</t>
+          <t>CTY-PATRICKSWELL-3</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Patrickswell – site 4</t>
+          <t>Patrickswell – site 3</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -6904,31 +6916,31 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.483</v>
+        <v>0.42</v>
       </c>
       <c r="E89" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Site status: Complete; Permission: 21873 - 5 units; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2560633 - 6 units  on 0.42; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-7</t>
+          <t>CTY-PATRICKSWELL-4</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Patrickswell – site 7</t>
+          <t>Patrickswell – site 4</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -6937,31 +6949,31 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>2.84</v>
+        <v>0.483</v>
       </c>
       <c r="E90" t="n">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 221318 - 51 units; Placement: area match (High)</t>
+          <t>Site status: Complete; Permission: 21873 - 5 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-8</t>
+          <t>CTY-PATRICKSWELL-7</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Patrickswell – site 8</t>
+          <t>Patrickswell – site 7</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -6970,31 +6982,31 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1.772</v>
+        <v>2.84</v>
       </c>
       <c r="E91" t="n">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Site status: Permission Granted; Permission: 2360144 - 44 units; Placement: area match (High)</t>
+          <t>Site status: Under Construction; Permission: 221318 - 51 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-9</t>
+          <t>CTY-PATRICKSWELL-8</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Patrickswell – site 9</t>
+          <t>Patrickswell – site 8</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -7003,31 +7015,31 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>2.398</v>
+        <v>1.772</v>
       </c>
       <c r="E92" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Site status: Under Construction; Permission: 19444 - 16 units, 181193 - 48 units; Placement: area match (High)</t>
+          <t>Site status: Permission Granted; Permission: 2360144 - 44 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-10</t>
+          <t>CTY-PATRICKSWELL-9</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Patrickswell – site 10</t>
+          <t>Patrickswell – site 9</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -7036,31 +7048,31 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.867</v>
+        <v>2.398</v>
       </c>
       <c r="E93" t="n">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Site status: No Permission Sought; Placement: area match (High)</t>
+          <t>Site status: Under Construction; Permission: 19444 - 16 units, 181193 - 48 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CTY-PATRICKSWELL-11</t>
+          <t>CTY-PATRICKSWELL-10</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Patrickswell – site 11</t>
+          <t>Patrickswell – site 10</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -7069,60 +7081,64 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.386</v>
+        <v>0.867</v>
       </c>
       <c r="E94" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Site status: Complete; Permission: 19689 - 8 units; Placement: area match (High)</t>
+          <t>Site status: No Permission Sought; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-U1</t>
+          <t>CTY-PATRICKSWELL-11</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Newcastle West – site U1</t>
+          <t>Patrickswell – site 11</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Town Centre</t>
+          <t>New Resi</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>3.815</v>
+        <v>0.386</v>
       </c>
       <c r="E95" t="n">
-        <v>0</v>
-      </c>
-      <c r="F95" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
+        </is>
+      </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Site status: Complete; Permission: 19689 - 8 units; Placement: area match (High)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CTY-NEWCASTLEWES-U2</t>
+          <t>CTY-NEWCASTLEWES-U1</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Newcastle West – site U2</t>
+          <t>Newcastle West – site U1</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -7134,227 +7150,243 @@
         <v>25.055</v>
       </c>
       <c r="E96" t="n">
-        <v>0</v>
-      </c>
-      <c r="F96" t="inlineStr"/>
+        <v>877</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Area x town average density for resi sites in the council audit (35/ha)</t>
+        </is>
+      </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-U1</t>
+          <t>CTY-NEWCASTLEWES-U2</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Rathkeale – site U1</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Enterprise and Employment</t>
-        </is>
-      </c>
+          <t>Newcastle West – site U2</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
-        <v>17.768</v>
+        <v>0.458</v>
       </c>
       <c r="E97" t="n">
-        <v>0</v>
-      </c>
-      <c r="F97" t="inlineStr"/>
+        <v>16</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Area x town average density for resi sites in the council audit (35/ha)</t>
+        </is>
+      </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-U2</t>
+          <t>CTY-NEWCASTLEWES-U3</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Rathkeale – site U2</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Enterprise and Employment</t>
-        </is>
-      </c>
+          <t>Newcastle West – site U3</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
       <c r="D98" t="n">
-        <v>14.728</v>
+        <v>0.831</v>
       </c>
       <c r="E98" t="n">
-        <v>0</v>
-      </c>
-      <c r="F98" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Area x town average density for resi sites in the council audit (35/ha)</t>
+        </is>
+      </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CTY-RATHKEALE-U3</t>
+          <t>CTY-NEWCASTLEWES-U4</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Rathkeale – site U3</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Enterprise and Employment</t>
-        </is>
-      </c>
+          <t>Newcastle West – site U4</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
-        <v>12.896</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="E99" t="n">
-        <v>0</v>
-      </c>
-      <c r="F99" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Area x town average density for resi sites in the council audit (35/ha)</t>
+        </is>
+      </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U1</t>
+          <t>CTY-NEWCASTLEWES-U5</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Askeaton – site U1</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Resi Service Site Phase 2</t>
-        </is>
-      </c>
+          <t>Newcastle West – site U5</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
       <c r="D100" t="n">
-        <v>0.86</v>
+        <v>5.045</v>
       </c>
       <c r="E100" t="n">
-        <v>0</v>
-      </c>
-      <c r="F100" t="inlineStr"/>
+        <v>177</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Area x town average density for resi sites in the council audit (35/ha)</t>
+        </is>
+      </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U2</t>
+          <t>CTY-RATHKEALE-U1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Askeaton – site U2</t>
+          <t>Rathkeale – site U1</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Resi Service Site Phase 1</t>
+          <t>Enterprise and Employment</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>1.182</v>
+        <v>17.768</v>
       </c>
       <c r="E101" t="n">
-        <v>0</v>
-      </c>
-      <c r="F101" t="inlineStr"/>
+        <v>391</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Area x town average density for resi sites in the council audit (22/ha)</t>
+        </is>
+      </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U3</t>
+          <t>CTY-RATHKEALE-U2</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Askeaton – site U3</t>
+          <t>Rathkeale – site U2</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Resi Development Area Phase 1</t>
+          <t>Enterprise and Employment</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>1.04</v>
+        <v>14.728</v>
       </c>
       <c r="E102" t="n">
-        <v>0</v>
-      </c>
-      <c r="F102" t="inlineStr"/>
+        <v>324</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Area x town average density for resi sites in the council audit (22/ha)</t>
+        </is>
+      </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U4</t>
+          <t>CTY-RATHKEALE-U3</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Askeaton – site U4</t>
+          <t>Rathkeale – site U3</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Resi Development Area Phase 1</t>
+          <t>Enterprise and Employment</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>7.428</v>
+        <v>12.896</v>
       </c>
       <c r="E103" t="n">
-        <v>0</v>
-      </c>
-      <c r="F103" t="inlineStr"/>
+        <v>284</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Area x town average density for resi sites in the council audit (22/ha)</t>
+        </is>
+      </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U5</t>
+          <t>CTY-ASKEATON-U1</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Askeaton – site U5</t>
+          <t>Askeaton – site U1</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -7363,27 +7395,31 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>2.098</v>
+        <v>0.86</v>
       </c>
       <c r="E104" t="n">
-        <v>0</v>
-      </c>
-      <c r="F104" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Area x town average density for serviced sites in the council audit (10/ha)</t>
+        </is>
+      </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CTY-ASKEATON-U6</t>
+          <t>CTY-ASKEATON-U2</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Askeaton – site U6</t>
+          <t>Askeaton – site U2</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -7392,159 +7428,163 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>2.684</v>
+        <v>1.182</v>
       </c>
       <c r="E105" t="n">
-        <v>0</v>
-      </c>
-      <c r="F105" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Area x town average density for serviced sites in the council audit (10/ha)</t>
+        </is>
+      </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Council site with no Excel row matched yet: fill in site number, density and capacity; Placement: council-supplied polygon, unmatched</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CTY-BALLINGARRY-1</t>
+          <t>CTY-ASKEATON-U3</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Ballingarry – site 1</t>
+          <t>Askeaton – site U3</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Resi Development Area Phase 1</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>1.75</v>
+        <v>1.04</v>
       </c>
       <c r="E106" t="n">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Area x town average density for resi sites in the council audit (22/ha)</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CTY-BALLINGARRY-2</t>
+          <t>CTY-ASKEATON-U4</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Ballingarry – site 2</t>
+          <t>Askeaton – site U4</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>Resi Development Area Phase 1</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>1.057</v>
+        <v>7.428</v>
       </c>
       <c r="E107" t="n">
-        <v>11</v>
+        <v>163</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Area x town average density for resi sites in the council audit (22/ha)</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CTY-BALLINGARRY-3</t>
+          <t>CTY-ASKEATON-U5</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Ballingarry – site 3</t>
+          <t>Askeaton – site U5</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>Resi Service Site Phase 2</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>2.903</v>
+        <v>2.098</v>
       </c>
       <c r="E108" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Area x town average density for serviced sites in the council audit (10/ha)</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>CTY-BRUREE-1</t>
+          <t>CTY-ASKEATON-U6</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Bruree – site 1</t>
+          <t>Askeaton – site U6</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Resi Service Site Phase 1</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1.15</v>
+        <v>2.684</v>
       </c>
       <c r="E109" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Area x town average density for serviced sites in the council audit (10/ha)</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon</t>
+          <t>Council site with no Excel row matched yet: site number to confirm; Placement: council-supplied polygon, unmatched</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>CTY-BRUREE-2</t>
+          <t>CTY-BALLINGARRY-1</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Bruree – site 2</t>
+          <t>Ballingarry – site 1</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -7553,14 +7593,14 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.247</v>
+        <v>1.75</v>
       </c>
       <c r="E110" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -7572,12 +7612,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CTY-BRUREE-3</t>
+          <t>CTY-BALLINGARRY-2</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Bruree – site 3</t>
+          <t>Ballingarry – site 2</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -7586,14 +7626,14 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.736</v>
+        <v>1.057</v>
       </c>
       <c r="E111" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -7605,28 +7645,28 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CTY-DROMCOLLIHER-1</t>
+          <t>CTY-BALLINGARRY-3</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 1</t>
+          <t>Ballingarry – site 3</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.8080000000000001</v>
+        <v>2.903</v>
       </c>
       <c r="E112" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -7638,12 +7678,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CTY-DROMCOLLIHER-2</t>
+          <t>CTY-BRUREE-1</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 2</t>
+          <t>Bruree – site 1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -7652,14 +7692,14 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.07099999999999999</v>
+        <v>1.15</v>
       </c>
       <c r="E113" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -7671,12 +7711,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CTY-DROMCOLLIHER-3</t>
+          <t>CTY-BRUREE-2</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 3</t>
+          <t>Bruree – site 2</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -7685,14 +7725,14 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.845</v>
+        <v>0.247</v>
       </c>
       <c r="E114" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -7704,12 +7744,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CTY-DROMCOLLIHER-4</t>
+          <t>CTY-BRUREE-3</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 4</t>
+          <t>Bruree – site 3</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -7718,14 +7758,14 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.773</v>
+        <v>0.736</v>
       </c>
       <c r="E115" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -7737,12 +7777,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CTY-FOYNES-1</t>
+          <t>CTY-DROMCOLLIHER-1</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Foynes – site 1</t>
+          <t>Dromcolliher – site 1</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -7751,14 +7791,14 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>3.497</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="E116" t="n">
-        <v>56</v>
+        <v>18</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -7770,28 +7810,28 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CTY-GLIN-1</t>
+          <t>CTY-DROMCOLLIHER-2</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Glin – site 1</t>
+          <t>Dromcolliher – site 2</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Mixed Use</t>
+          <t>New Residential</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>1.613</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="E117" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -7803,12 +7843,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CTY-GLIN-2</t>
+          <t>CTY-DROMCOLLIHER-3</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Glin – site 2</t>
+          <t>Dromcolliher – site 3</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -7817,14 +7857,14 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.527</v>
+        <v>0.845</v>
       </c>
       <c r="E118" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -7836,12 +7876,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CTY-GLIN-3</t>
+          <t>CTY-DROMCOLLIHER-4</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Glin – site 3</t>
+          <t>Dromcolliher – site 4</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -7850,14 +7890,14 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.965</v>
+        <v>0.773</v>
       </c>
       <c r="E119" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -7869,12 +7909,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CTY-GLIN-4</t>
+          <t>CTY-FOYNES-1</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Glin – site 4</t>
+          <t>Foynes – site 1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -7883,14 +7923,14 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>1.25</v>
+        <v>3.497</v>
       </c>
       <c r="E120" t="n">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -7902,28 +7942,28 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CTY-HOSPITAL-5</t>
+          <t>CTY-GLIN-1</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Hospital – site 5</t>
+          <t>Glin – site 1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Enterprise &amp; Employment</t>
+          <t>Mixed Use</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>2.675</v>
+        <v>1.613</v>
       </c>
       <c r="E121" t="n">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Estimate (council audit recorded no capacity): developable area x density</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -7935,12 +7975,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CTY-PALLASGREEN-2</t>
+          <t>CTY-GLIN-2</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Pallasgreen – site 2</t>
+          <t>Glin – site 2</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -7949,14 +7989,14 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>1.424</v>
+        <v>0.527</v>
       </c>
       <c r="E122" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -7968,28 +8008,28 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>CTY-PALLASGREEN-1</t>
+          <t>CTY-GLIN-3</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Pallasgreen – site 1</t>
+          <t>Glin – site 3</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>New Residential</t>
+          <t>Residential Serviced Sites</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>0.613</v>
+        <v>0.965</v>
       </c>
       <c r="E123" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -8001,28 +8041,28 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CTY-PALLASGREEN-3</t>
+          <t>CTY-GLIN-4</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Pallasgreen – site 3</t>
+          <t>Glin – site 4</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>New Residential</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1.07</v>
+        <v>1.25</v>
       </c>
       <c r="E124" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -8034,64 +8074,196 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CTY-PALLASKENRY-4</t>
+          <t>CTY-HOSPITAL-5</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Pallaskenry – site 4</t>
+          <t>Hospital – site 5</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Residential Serviced Sites</t>
+          <t>Enterprise &amp; Employment</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>0.271</v>
+        <v>2.675</v>
       </c>
       <c r="E125" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
+          <t>Area x town average density for resi sites in the council audit (22/ha)</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Placement: 2022 polygon; clipped by consent 24352</t>
+          <t>Placement: 2022 polygon</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
+          <t>CTY-PALLASGREEN-2</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Pallasgreen – site 2</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>1.424</v>
+      </c>
+      <c r="E126" t="n">
+        <v>31</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>CTY-PALLASGREEN-1</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Pallasgreen – site 1</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>New Residential</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>0.613</v>
+      </c>
+      <c r="E127" t="n">
+        <v>14</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>CTY-PALLASGREEN-3</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Pallasgreen – site 3</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E128" t="n">
+        <v>11</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>CTY-PALLASKENRY-4</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Pallaskenry – site 4</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Residential Serviced Sites</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="E129" t="n">
+        <v>3</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Placement: 2022 polygon; clipped by consent 24352</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
           <t>CTY-PALLASKENRY-3</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
+      <c r="B130" t="inlineStr">
         <is>
           <t>Pallaskenry – site 3</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>New Residential</t>
         </is>
       </c>
-      <c r="D126" t="n">
+      <c r="D130" t="n">
         <v>0.753</v>
       </c>
-      <c r="E126" t="n">
+      <c r="E130" t="n">
         <v>17</v>
       </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>Council county audit: area x density (County audit 2022 (not in the May 2026 Excel))</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Council area x density (County audit 2022 (not in the May 2026 Excel))</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
         <is>
           <t>Placement: 2022 polygon</t>
         </is>
@@ -10461,7 +10633,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Council county audit capacity (Council capacity audit Excel (May 2026))</t>
+          <t>Council capacity (Council capacity audit Excel (May 2026))</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Register: merge non-city parcel review (208 accepted, 3 removed)
Review stored as inputs (status by parcel_id, matched by shape where IDs move; removed land and permissions kept out).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-26 15:46</t>
+          <t>2026-10-26 16:54</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>452 parcels</t>
+          <t>449 parcels</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>263 permissions</t>
+          <t>262 permissions</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>permission units 11,043 vs parcel buckets 11,043; max parcel imbalance 0.00</t>
+          <t>permission units 11,022 vs parcel buckets 11,022; max parcel imbalance 0.00</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>supply GeoPackage and register hold the same permissions and units</t>
+          <t>supply GeoPackage and register hold the same permissions and units (less review removals)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>263 vs 263 permissions</t>
+          <t>263 vs 262 permissions; 1 removed at review</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{'Inside catchment': 364, 'Rest of county': 46, 'Edge of settlement (within 500 m)': 32, 'Zoned in': 9, 'Named in scheme, within 2 km': 1}</t>
+          <t>{'Inside catchment': 363, 'Rest of county': 45, 'Edge of settlement (within 500 m)': 32, 'Zoned in': 8, 'Named in scheme, within 2 km': 1}</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>236 of 242 references found live (26/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
+          <t>235 of 241 references found live (26/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
         </is>
       </c>
     </row>
@@ -1389,11 +1389,11 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1,120 homes in 8 plan areas: ask the council for audits of these towns</t>
+          <t>1,109 homes in 8 plan areas: ask the council for audits of these towns</t>
         </is>
       </c>
     </row>
@@ -3948,13 +3948,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>0.947</v>
+        <v>0.469</v>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -8280,7 +8280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8318,13 +8318,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1424651</t>
+          <t>1034286</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>19149</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
@@ -8336,14 +8340,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1438055</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+          <t>1424651</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>left_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1438055</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
         <is>
           <t>left_only</t>
         </is>
@@ -10357,7 +10379,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PC-228017</t>
+          <t>PC-188012</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">

</xml_diff>

<commit_message>
Register: drop review columns (all accepted), permissions count as tier 1 serviced, standard parcel descriptions
- local_name is now a standard description (place, homes, scheme type); original heading kept in source_name
- parcels with a live permission are classed Serviced (tier 1)
- review status/notes columns and review-matching inputs removed; review removals still applied

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-27 10:00</t>
+          <t>2026-10-27 10:16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 1</t>
+          <t>Abbeyfeale: council audit site 1, 19 homes capacity, brownfield</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3985,7 +3985,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 10</t>
+          <t>Abbeyfeale: council audit site 10, 5 homes capacity, infill</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 2</t>
+          <t>Abbeyfeale: council audit site 2, 35 homes capacity, brownfield</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 3</t>
+          <t>Abbeyfeale: council audit site 3, 9 homes capacity, brownfield</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 4</t>
+          <t>Abbeyfeale: council audit site 4, 8 homes capacity, infill</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4117,7 +4117,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 5</t>
+          <t>Abbeyfeale: council audit site 5, 92 homes capacity, greenfield; 68 homes permitted</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -4150,7 +4150,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 6</t>
+          <t>Abbeyfeale: council audit site 6, 59 homes capacity, infill</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 7</t>
+          <t>Abbeyfeale: council audit site 7, 10 homes capacity, infill</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 8</t>
+          <t>Abbeyfeale: council audit site 8, 31 homes capacity, brownfield</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Abbeyfeale – site 9</t>
+          <t>Abbeyfeale: council audit site 9, 15 homes capacity, infill</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4282,7 +4282,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Askeaton – site 1</t>
+          <t>Askeaton: council audit site 1, 27 homes capacity, infill</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -4315,7 +4315,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Askeaton – site 10</t>
+          <t>Askeaton: council audit site 10, 104 homes capacity, infill</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Askeaton – site 11</t>
+          <t>Askeaton: council audit site 11, 34 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Askeaton – site 2</t>
+          <t>Askeaton: council audit site 2, 15 homes capacity, infill</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Askeaton – site 3</t>
+          <t>Askeaton: council audit site 3, 93 homes capacity, infill</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Askeaton – site 4</t>
+          <t>Askeaton: council audit site 4, 35 homes capacity, infill</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -4480,7 +4480,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Askeaton – site 5</t>
+          <t>Askeaton: council audit site 5, 23 homes capacity, infill</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -4513,7 +4513,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Askeaton – site 6</t>
+          <t>Askeaton: council audit site 6, 10 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Askeaton – site 7</t>
+          <t>Askeaton: council audit site 7, 13 homes capacity, infill</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Askeaton – site 8</t>
+          <t>Askeaton: council audit site 8, 6 homes capacity, infill</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4612,7 +4612,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Askeaton – site 9</t>
+          <t>Askeaton: council audit site 9, 25 homes capacity, infill</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Caherconlish – site 1</t>
+          <t>Caherconlish: council audit site 1, 79 homes capacity, infill</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4678,7 +4678,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Caherconlish – site 2</t>
+          <t>Caherconlish: council audit site 2, 10 homes capacity, infill</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4711,7 +4711,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Caherconlish – site 3</t>
+          <t>Caherconlish: council audit site 3, 5 homes capacity, infill</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Caherconlish – site 4</t>
+          <t>Caherconlish: council audit site 4, 46 homes capacity, infill</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Caherconlish – site 5</t>
+          <t>Caherconlish: council audit site 5, 21 homes capacity, infill</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Caherconlish – site 6</t>
+          <t>Caherconlish: council audit site 6, 0 homes capacity, infill; 9 homes permitted</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4843,7 +4843,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Caherconlish – site 7</t>
+          <t>Caherconlish: council audit site 7, 130 homes capacity</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Cappamore – site 1</t>
+          <t>Cappamore: council audit site 1, 29 homes capacity, greenfield; 17 homes permitted</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cappamore – site 2</t>
+          <t>Cappamore: council audit site 2, 7 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -4942,7 +4942,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Cappamore – site 3</t>
+          <t>Cappamore: council audit site 3, 22 homes capacity, infill; 22 homes permitted</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -4975,7 +4975,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Cappamore – site 4</t>
+          <t>Cappamore: council audit site 4, 6 homes capacity, infill; 10 homes permitted</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Cappamore – site 5</t>
+          <t>Cappamore: council audit site 5, 4 homes capacity, infill; 7 homes permitted</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5041,7 +5041,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cappamore – site 6</t>
+          <t>Cappamore: council audit site 6, 3 homes capacity, infill</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5074,7 +5074,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Castleconnell – site 1</t>
+          <t>Castleconnell: council audit site 1, 6 homes capacity, infill</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5107,7 +5107,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Castleconnell – site 10</t>
+          <t>Castleconnell: council audit site 10, 88 homes capacity</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5140,7 +5140,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Castleconnell – site 2</t>
+          <t>Castleconnell: council audit site 2, 14 homes capacity, infill</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Castleconnell – site 3</t>
+          <t>Castleconnell: council audit site 3, 14 homes capacity, infill</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Castleconnell – site 4</t>
+          <t>Castleconnell: council audit site 4, 134 homes capacity, infill; 74 homes permitted</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Castleconnell – site 5a</t>
+          <t>Castleconnell: council audit site 5a, 9 homes capacity, infill</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -5272,7 +5272,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Castleconnell – site 5b</t>
+          <t>Castleconnell: council audit site 5b, 2 homes capacity, infill</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Castleconnell – site 6</t>
+          <t>Castleconnell: council audit site 6, 11 homes capacity, infill</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5338,7 +5338,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Castleconnell – site 7</t>
+          <t>Castleconnell: council audit site 7, 14 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Castleconnell – site 8</t>
+          <t>Castleconnell: council audit site 8, 16 homes capacity, infill</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Castleconnell – site 9</t>
+          <t>Castleconnell: council audit site 9, 148 homes capacity</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -5437,7 +5437,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Croom – site 1</t>
+          <t>Croom: council audit site 1, 11 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Croom – site 2</t>
+          <t>Croom: council audit site 2, 65 homes capacity, infill; 51 homes permitted</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5503,7 +5503,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Croom – site 3</t>
+          <t>Croom: council audit site 3, 4 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Croom – site 4</t>
+          <t>Croom: council audit site 4, 12 homes capacity, infill; 16 homes permitted</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Croom – site 5</t>
+          <t>Croom: council audit site 5, 89 homes capacity, infill</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -5602,7 +5602,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Croom – site 6</t>
+          <t>Croom: council audit site 6, 44 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -5635,7 +5635,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Croom – site 7</t>
+          <t>Croom: council audit site 7, 27 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Croom – site 8</t>
+          <t>Croom: council audit site 8, 7 homes capacity, infill; 10 homes permitted</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -5701,7 +5701,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Kilmallock – site 1.1</t>
+          <t>Kilmallock: council audit site 1.1, 61 homes capacity, infill</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -5734,7 +5734,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Kilmallock – site 1.2</t>
+          <t>Kilmallock: council audit site 1.2, 24 homes capacity, infill; 28 homes permitted</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Kilmallock – site 10.1</t>
+          <t>Kilmallock: council audit site 10.1, 32 homes capacity, infill</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -5800,7 +5800,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Kilmallock – site 10.2</t>
+          <t>Kilmallock: council audit site 10.2, 24 homes capacity, infill; 42 homes permitted</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -5833,7 +5833,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Kilmallock – site 10.3</t>
+          <t>Kilmallock: council audit site 10.3, 37 homes capacity, infill</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -5866,7 +5866,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Kilmallock – site 2</t>
+          <t>Kilmallock: council audit site 2, 38 homes capacity, infill</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Kilmallock – site 3</t>
+          <t>Kilmallock: council audit site 3, 19 homes capacity</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -5928,7 +5928,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Kilmallock – site 4</t>
+          <t>Kilmallock: council audit site 4, 126 homes capacity</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Kilmallock – site 5</t>
+          <t>Kilmallock: council audit site 5, 44 homes capacity</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -5986,7 +5986,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Kilmallock – site 6</t>
+          <t>Kilmallock: council audit site 6, 133 homes capacity</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Kilmallock – site 7</t>
+          <t>Kilmallock: council audit site 7, 112 homes capacity</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -6044,7 +6044,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Kilmallock – site 8</t>
+          <t>Kilmallock: council audit site 8, 37 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Kilmallock – site 9.1</t>
+          <t>Kilmallock: council audit site 9.1, 35 homes capacity, infill</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Kilmallock – site 9.2</t>
+          <t>Kilmallock: council audit site 9.2, 83 homes capacity, infill</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -6143,7 +6143,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Newcastle West – site 1</t>
+          <t>Newcastle West: council audit site 1, 16 homes capacity, brownfield</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Newcastle West – site 10</t>
+          <t>Newcastle West: council audit site 10, 42 homes capacity, infill</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -6209,7 +6209,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Newcastle West – site 11</t>
+          <t>Newcastle West: council audit site 11, 1068 homes capacity</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Newcastle West – site 12</t>
+          <t>Newcastle West: council audit site 12, 28 homes capacity, infill</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -6275,7 +6275,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Newcastle West – site 13</t>
+          <t>Newcastle West: council audit site 13, 74 homes capacity, infill; 14 homes permitted</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Newcastle West – site 14</t>
+          <t>Newcastle West: council audit site 14, 46 homes capacity, infill; 31 homes permitted</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Newcastle West – site 15</t>
+          <t>Newcastle West: council audit site 15, 30 homes capacity, infill</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Newcastle West – site 16</t>
+          <t>Newcastle West: council audit site 16, 21 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Newcastle West – site 17</t>
+          <t>Newcastle West: council audit site 17, 39 homes capacity, infill</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Newcastle West – site 18</t>
+          <t>Newcastle West: council audit site 18, 877 homes capacity</t>
         </is>
       </c>
       <c r="C78" t="inlineStr"/>
@@ -6469,7 +6469,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Newcastle West – site 19</t>
+          <t>Newcastle West: council audit site 19, 190 homes capacity</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Newcastle West – site 2</t>
+          <t>Newcastle West: council audit site 2, 13 homes capacity, infill</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Newcastle West – site 3</t>
+          <t>Newcastle West: council audit site 3, 40 homes capacity, infill</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -6564,7 +6564,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Newcastle West – site 4</t>
+          <t>Newcastle West: council audit site 4, 26 homes capacity, infill</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -6597,7 +6597,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Newcastle West – site 5</t>
+          <t>Newcastle West: council audit site 5, 438 homes capacity, infill; 93 homes permitted</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -6630,7 +6630,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Newcastle West – site 6</t>
+          <t>Newcastle West: council audit site 6, 0 homes capacity, greenfield; 53 homes permitted</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -6663,7 +6663,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Newcastle West – site 7</t>
+          <t>Newcastle West: council audit site 7, 10 homes capacity, brownfield</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Newcastle West – site 8</t>
+          <t>Newcastle West: council audit site 8, 14 homes capacity, brownfield</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -6729,7 +6729,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Newcastle West – site 9</t>
+          <t>Newcastle West: council audit site 9, 66 homes capacity, infill</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Rathkeale – site 1</t>
+          <t>Rathkeale: council audit site 1, 9 homes capacity, infill</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -6795,7 +6795,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Rathkeale – site 10</t>
+          <t>Rathkeale: council audit site 10, 18 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Rathkeale – site 11</t>
+          <t>Rathkeale: council audit site 11, 391 homes capacity</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Rathkeale – site 12</t>
+          <t>Rathkeale: council audit site 12, 324 homes capacity</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Rathkeale – site 13</t>
+          <t>Rathkeale: council audit site 13, 284 homes capacity</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Rathkeale – site 2</t>
+          <t>Rathkeale: council audit site 2, 23 homes capacity, infill</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -6960,7 +6960,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Rathkeale – site 3</t>
+          <t>Rathkeale: council audit site 3, 34 homes capacity, infill</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -6993,7 +6993,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Rathkeale – site 4</t>
+          <t>Rathkeale: council audit site 4, 8 homes capacity, infill</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -7026,7 +7026,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Rathkeale – site 5</t>
+          <t>Rathkeale: council audit site 5, 13 homes capacity, infill</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -7059,7 +7059,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Rathkeale – site 6</t>
+          <t>Rathkeale: council audit site 6, 18 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -7092,7 +7092,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Rathkeale – site 7</t>
+          <t>Rathkeale: council audit site 7, 28 homes capacity, infill</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -7125,7 +7125,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Rathkeale – site 8</t>
+          <t>Rathkeale: council audit site 8, 30 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Rathkeale – site 9</t>
+          <t>Rathkeale: council audit site 9, 4 homes capacity, infill</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Adare – site 1a</t>
+          <t>Adare: council audit site 1a, 24 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Adare – site 5</t>
+          <t>Adare: council audit site 5, 37 homes capacity, infill</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Adare – site 6</t>
+          <t>Adare: council audit site 6, 7 homes capacity, infill</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Adare – site 8</t>
+          <t>Adare: council audit site 8, 12 homes capacity, brownfield</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Bruff – site 1</t>
+          <t>Bruff: council audit site 1, 72 homes capacity, greenfield; 74 homes permitted</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -7356,7 +7356,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Bruff – site 2</t>
+          <t>Bruff: council audit site 2, 15 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -7389,7 +7389,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Bruff – site 4</t>
+          <t>Bruff: council audit site 4, 5 homes capacity, infill</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Bruff – site 3</t>
+          <t>Bruff: council audit site 3, 14 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Hospital – site 1</t>
+          <t>Hospital: council audit site 1, 14 homes capacity, infill</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -7488,7 +7488,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Hospital – site 2</t>
+          <t>Hospital: council audit site 2, 22 homes capacity, brownfield</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Hospital – site 3</t>
+          <t>Hospital: council audit site 3, 15 homes capacity, infill</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Hospital – site 4</t>
+          <t>Hospital: council audit site 4, 10 homes capacity, infill</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Kilfinane – site 1</t>
+          <t>Kilfinnane: council audit site 1, 9 homes capacity, greenfield; 10 homes permitted</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -7620,7 +7620,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Kilfinane – site 2</t>
+          <t>Kilfinnane: council audit site 2, 7 homes capacity, infill</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -7653,7 +7653,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Kilfinane – site 3</t>
+          <t>Kilfinnane: council audit site 3, 18 homes capacity, infill</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Kilfinane – site 4</t>
+          <t>Kilfinnane: council audit site 4, 16 homes capacity, infill</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -7719,7 +7719,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Kilfinane – site 5</t>
+          <t>Kilfinnane: council audit site 5, 15 homes capacity, infill</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -7752,7 +7752,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Murroe – site 1</t>
+          <t>Moroe: council audit site 1, 40 homes capacity, infill</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Murroe – site 2</t>
+          <t>Moroe: council audit site 2, 22 homes capacity, infill</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -7818,7 +7818,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Murroe – site 3</t>
+          <t>Moroe: council audit site 3, 24 homes capacity, infill; 32 homes permitted</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Murroe – site 4</t>
+          <t>Moroe: council audit site 4, 19 homes capacity, infill</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Patrickswell – site 1</t>
+          <t>Patrickswell: council audit site 1, 90 homes capacity, greenfield; 103 homes permitted</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -7917,7 +7917,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Patrickswell – site 2</t>
+          <t>Patrickswell: council audit site 2, 65 homes capacity, greenfield</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -7950,7 +7950,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Patrickswell – site 14</t>
+          <t>Patrickswell: council audit site 14, 48 homes capacity, greenfield; 90 homes permitted</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Patrickswell – site 17</t>
+          <t>Patrickswell: council audit site 17, 4 homes capacity, infill</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Patrickswell – site 3</t>
+          <t>Patrickswell: council audit site 3, 9 homes capacity, infill; 6 homes permitted</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -8049,7 +8049,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Patrickswell – site 4</t>
+          <t>Patrickswell: council audit site 4, 11 homes capacity, infill; 9 homes permitted</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -8082,7 +8082,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Patrickswell – site 7</t>
+          <t>Patrickswell: council audit site 7, 62 homes capacity, greenfield; 52 homes permitted</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Patrickswell – site 8</t>
+          <t>Patrickswell: council audit site 8, 39 homes capacity, brownfield; 41 homes permitted</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Patrickswell – site 9</t>
+          <t>Patrickswell: council audit site 9, 53 homes capacity, infill; 63 homes permitted</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Patrickswell – site 10</t>
+          <t>Patrickswell: council audit site 10, 19 homes capacity, infill</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Patrickswell – site 11</t>
+          <t>Patrickswell: council audit site 11, 8 homes capacity, infill; 9 homes permitted</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -8247,7 +8247,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Ballingarry – site 1</t>
+          <t>Ballingarry (rest of county): council audit site 1, 38 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -8280,7 +8280,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Ballingarry – site 2</t>
+          <t>Ballingarry (rest of county): council audit site 2, 11 homes capacity</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -8313,7 +8313,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Ballingarry – site 3</t>
+          <t>Ballingarry (rest of county): council audit site 3, 29 homes capacity</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -8346,7 +8346,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Bruree – site 1</t>
+          <t>Bruree (rest of county): council audit site 1, 25 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -8379,7 +8379,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Bruree – site 2</t>
+          <t>Bruree (rest of county): council audit site 2, 5 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -8412,7 +8412,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Bruree – site 3</t>
+          <t>Bruree (rest of county): council audit site 3, 7 homes capacity</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 1</t>
+          <t>Dromcolliher (rest of county): council audit site 1, 18 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -8478,7 +8478,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 2</t>
+          <t>Dromcolliher (rest of county): council audit site 2, 2 homes capacity</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 3</t>
+          <t>Dromcolliher (rest of county): council audit site 3, 19 homes capacity</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Dromcolliher – site 4</t>
+          <t>Dromcolliher (rest of county): council audit site 4, 8 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Foynes – site 1</t>
+          <t>Foynes (rest of county): council audit site 1, 56 homes capacity</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -8610,7 +8610,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Glin – site 1</t>
+          <t>Glin (rest of county): council audit site 1, 36 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -8643,7 +8643,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Glin – site 2</t>
+          <t>Glin (rest of county): council audit site 2, 12 homes capacity; 10 homes permitted</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -8676,7 +8676,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Glin – site 3</t>
+          <t>Glin (rest of county): council audit site 3, 10 homes capacity</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -8709,7 +8709,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Glin – site 4</t>
+          <t>Glin (rest of county): council audit site 4, 27 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -8742,7 +8742,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Hospital – site 5</t>
+          <t>Hospital: council audit site 5, 59 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Pallasgreen – site 2</t>
+          <t>Pallasgreen (rest of county): council audit site 2, 31 homes capacity, infill/brownfield; 6 homes permitted</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Pallasgreen – site 1</t>
+          <t>Pallasgreen (rest of county): council audit site 1, 14 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Pallasgreen – site 3</t>
+          <t>Pallasgreen (rest of county): council audit site 3, 11 homes capacity, infill/brownfield</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -8874,7 +8874,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Pallaskenry – site 4</t>
+          <t>Pallaskenry (rest of county): council audit site 4, 3 homes capacity</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -8907,7 +8907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Pallaskenry – site 3</t>
+          <t>Pallaskenry (rest of county): council audit site 3, 17 homes capacity</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -11242,7 +11242,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Garryowen</t>
+          <t>Singland/Garryowen: council audit site 84, 20 homes capacity, brownfield; 30 homes permitted</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>City Centre</t>
+          <t>City Centre: council audit site 106, 36 homes capacity, brownfield; 36 homes permitted</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -11304,7 +11304,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Caherconlish – site 6</t>
+          <t>Caherconlish: council audit site 6, 0 homes capacity, infill; 9 homes permitted</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -11335,7 +11335,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Newcastle West – site 6</t>
+          <t>Newcastle West: council audit site 6, 0 homes capacity, greenfield; 53 homes permitted</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -11397,7 +11397,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Northside</t>
+          <t>Caherdavin: council audit site 12, 73 homes capacity, greenfield; 115 homes permitted</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -11415,7 +11415,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Corbally</t>
+          <t>Corbally/Grove Island: council audit site 30, 21 homes capacity, infill; 25 homes permitted</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -11433,7 +11433,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Garryowen</t>
+          <t>Singland/Garryowen: council audit site 49, 11 homes capacity, infill; 25 homes permitted</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -11451,7 +11451,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Castletroy</t>
+          <t>Castletroy/Annacotty: council audit site 53, 108 homes capacity, infill; 196 homes permitted</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -11469,7 +11469,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Castletroy</t>
+          <t>Castletroy/Annacotty: council audit site 56, 123 homes capacity, infill; 146 homes permitted</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Castletroy</t>
+          <t>Castletroy/Annacotty: council audit site 71, 141 homes capacity, infill; 465 homes permitted</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -11505,7 +11505,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Castletroy</t>
+          <t>Castletroy/Annacotty: council audit site 72, 216 homes capacity, greenfield; 260 homes permitted</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Garryowen</t>
+          <t>Southhill: council audit site 74, 19 homes capacity, infill; 31 homes permitted</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -11541,7 +11541,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Garryowen</t>
+          <t>Southhill: council audit site 76, 245 homes capacity, brownfield; 403 homes permitted</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -11559,7 +11559,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Garryowen</t>
+          <t>Singland/Garryowen: council audit site 83, 14 homes capacity, brownfield; 44 homes permitted</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -11577,7 +11577,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Garryowen</t>
+          <t>Singland/Garryowen: council audit site 84, 20 homes capacity, brownfield; 30 homes permitted</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -11593,7 +11593,11 @@
           <t>CITY-113</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Southhill: council audit site 113, 9 homes capacity, infill; 10 homes permitted</t>
+        </is>
+      </c>
       <c r="C13" t="n">
         <v>9</v>
       </c>
@@ -11609,7 +11613,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dock Rd</t>
+          <t>Ballinacurra: council audit site 133, 55 homes capacity, infill; 371 homes permitted</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -11627,7 +11631,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dooradoyle</t>
+          <t>Dooradoyle: council audit site 149, 33 homes capacity, infill; 250 homes permitted</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -11645,7 +11649,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Caherconlish – site 6</t>
+          <t>Caherconlish: council audit site 6, 0 homes capacity, infill; 9 homes permitted</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -11663,7 +11667,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cappamore – site 4</t>
+          <t>Cappamore: council audit site 4, 6 homes capacity, infill; 10 homes permitted</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -11681,7 +11685,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cappamore – site 5</t>
+          <t>Cappamore: council audit site 5, 4 homes capacity, infill; 7 homes permitted</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -11699,7 +11703,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Croom – site 4</t>
+          <t>Croom: council audit site 4, 12 homes capacity, infill; 16 homes permitted</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -11717,7 +11721,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Croom – site 8</t>
+          <t>Croom: council audit site 8, 7 homes capacity, infill; 10 homes permitted</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -11735,7 +11739,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kilmallock – site 1.2</t>
+          <t>Kilmallock: council audit site 1.2, 24 homes capacity, infill; 28 homes permitted</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -11753,7 +11757,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Kilmallock – site 10.2</t>
+          <t>Kilmallock: council audit site 10.2, 24 homes capacity, infill; 42 homes permitted</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -11771,7 +11775,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Newcastle West – site 6</t>
+          <t>Newcastle West: council audit site 6, 0 homes capacity, greenfield; 53 homes permitted</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -11789,7 +11793,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kilfinane – site 1</t>
+          <t>Kilfinnane: council audit site 1, 9 homes capacity, greenfield; 10 homes permitted</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -11807,7 +11811,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Murroe – site 3</t>
+          <t>Moroe: council audit site 3, 24 homes capacity, infill; 32 homes permitted</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -11825,7 +11829,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Patrickswell – site 1</t>
+          <t>Patrickswell: council audit site 1, 90 homes capacity, greenfield; 103 homes permitted</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -11843,7 +11847,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Patrickswell – site 14</t>
+          <t>Patrickswell: council audit site 14, 48 homes capacity, greenfield; 90 homes permitted</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -11861,7 +11865,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Patrickswell – site 9</t>
+          <t>Patrickswell: council audit site 9, 53 homes capacity, infill; 63 homes permitted</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -11879,7 +11883,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Patrickswell – site 11</t>
+          <t>Patrickswell: council audit site 11, 8 homes capacity, infill; 9 homes permitted</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -11943,7 +11947,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>€8.6m - Staff Accommodation/8Apartments, Adare</t>
+          <t>Adare: 28 homes, apartments – private scheme</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -11969,7 +11973,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>€7m - Residential Development, Condell Road</t>
+          <t>Caherdavin: 43 homes, houses – social scheme (council)</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -11995,7 +11999,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>€5.4m - Patricks Well Housing Development, Mungret</t>
+          <t>Dooradoyle: 54 homes, houses and apartments – private scheme</t>
         </is>
       </c>
       <c r="C4" t="n">

</xml_diff>

<commit_message>
Register: manual capacity overrides (CITY-107 masterplanned city-centre site = 2,500 homes)
Overrides live in inputs/manual_capacity.csv with reason and date; flagged in capacity_manual, capacity_basis and notes,
and listed in validation check P6.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-27 10:27</t>
+          <t>2026-10-27 10:39</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1209,11 +1209,11 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>25 hand-entered items; 0 mix rows not adding up; 0 added schemes no longer granted</t>
+          <t>29 hand-entered items; 0 mix rows not adding up; 0 added schemes no longer granted</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2831,68 +2831,68 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Unit mix from planning file</t>
+          <t>Manual capacity override</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>22840</t>
+          <t>CITY-107</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Planner's report (decision) – development contributions schedule; beds 93 houses+apts 93 total 93</t>
+          <t>2,500 homes, set 2026-10-27 by Analyst: Masterplanned city-centre mixed-use site (about 60 ha); no application yet; earmarked for 2,500 homes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Unit mix from planning file</t>
+          <t>Parcel removed at review</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ABP-307631</t>
+          <t>ZN-Kilmallock-002</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>An Bord Pleanála inspector's report (unit mix table); beds 200 houses+apts 200 total 200</t>
+          <t>this is a leftover green space. units complete</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Unit mix from planning file</t>
+          <t>Parcel removed at review</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>19970</t>
+          <t>ZN-Kilmallock-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>An Bord Pleanála inspector's report 307386-20 (scheme as revised at further information); beds 92 houses+apts 92 total 92</t>
+          <t>this is a leftover green space. units complete</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Unit mix from planning file</t>
+          <t>Parcel removed at review</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2560156</t>
+          <t>PC-19149</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Planner's report (unit-by-unit schedule; council stage – decision upheld on appeal ACP-323113-25); beds 63 houses+apts 63 total 63</t>
+          <t>incorrect application</t>
         </is>
       </c>
     </row>
@@ -2904,12 +2904,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>221318</t>
+          <t>22840</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Schedule of accommodation (application); beds 52 houses+apts 52 total 52</t>
+          <t>Planner's report (decision) – development contributions schedule; beds 93 houses+apts 93 total 93</t>
         </is>
       </c>
     </row>
@@ -2921,12 +2921,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2360144</t>
+          <t>ABP-307631</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Planner's report (unit-by-unit schedule); beds 41 houses+apts 41 total 41</t>
+          <t>An Bord Pleanála inspector's report (unit mix table); beds 200 houses+apts 200 total 200</t>
         </is>
       </c>
     </row>
@@ -2938,12 +2938,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2560653</t>
+          <t>19970</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Housing quality assessment (submitted with further information); beds 42 houses+apts 42 total 42</t>
+          <t>An Bord Pleanála inspector's report 307386-20 (scheme as revised at further information); beds 92 houses+apts 92 total 92</t>
         </is>
       </c>
     </row>
@@ -2955,12 +2955,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>181193</t>
+          <t>2560156</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Planner's report on 25/60133 (amendment to 18/1193): 33 x 3-bed and 16 x 2-bed granted; 6 houses changed 2-bed to 3-bed; beds 49 houses+apts 49 total 49</t>
+          <t>Planner's report (unit-by-unit schedule; council stage – decision upheld on appeal ACP-323113-25); beds 63 houses+apts 63 total 63</t>
         </is>
       </c>
     </row>
@@ -2972,10 +2972,78 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>221318</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Schedule of accommodation (application); beds 52 houses+apts 52 total 52</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Unit mix from planning file</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2360144</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Planner's report (unit-by-unit schedule); beds 41 houses+apts 41 total 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Unit mix from planning file</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2560653</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Housing quality assessment (submitted with further information); beds 42 houses+apts 42 total 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Unit mix from planning file</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>181193</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Planner's report on 25/60133 (amendment to 18/1193): 33 x 3-bed and 16 x 2-bed granted; 6 houses changed 2-bed to 3-bed; beds 49 houses+apts 49 total 49</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Unit mix from planning file</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>2460788</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Planning &amp; design statement – development accommodation schedule; beds 42 houses+apts 42 total 42</t>
         </is>

</xml_diff>

<commit_message>
Opportunity sites: 14 new sites filled (Kilfinnane, Murroe, city); CITY-107 split 50/50 City Centre / Singland in needs model
- opportunity register rebuilt from the returned copy, keeping all entries and IDs
- manual_capacity.csv gains catchment_split; needs-model land tab shares CITY-107 land and homes 50/50
- needs model rebuilt (zoned land vs need, opportunity sites & options)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-27 16:07</t>
+          <t>2026-10-28 10:30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>235 of 241 references found live (27/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
+          <t>235 of 241 references found live (28/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2,500 homes, set 2026-10-27 by Analyst: Masterplanned city-centre mixed-use site (about 60 ha); no application yet; earmarked for 2,500 homes</t>
+          <t>2,500 homes, set 2026-10-27 by Analyst: Masterplanned city-centre mixed-use site (about 60 ha); no application yet; earmarked for 2,500 homes. Half the site and half the homes lie in Singland/Garryowen: split 50/50 with City Centre in the needs model</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rerun validation report on the netted register (18 PASS, 12 WARN)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzU6RZjdYh3MCXCEtKHHfb
</commit_message>
<xml_diff>
--- a/limerick_pipeline/register/Validation_Report.xlsx
+++ b/limerick_pipeline/register/Validation_Report.xlsx
@@ -474,7 +474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-28 10:30</t>
+          <t>2026-10-30 12:59</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>235 of 241 references found live (28/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
+          <t>235 of 241 references found live (30/10/2026); 6 outside the dataset's coverage (Part 8 / pre-2017)</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -2430,7 +2430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2468,61 +2468,113 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1402906</t>
+          <t>1350852</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2560399</t>
+          <t>2460570</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">€16.4m - Residential Development </t>
+          <t>€4.5m - Apartment Development, Limerick City</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>Permitted – not started</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
+      <c r="F2" s="1" t="n">
+        <v>46316</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>1402906</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2560399</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">€16.4m - Residential Development </t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>76</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>46303</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>1166991</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>21630</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>€10.8m - Residential Development, Croom</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>51</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Permitted – not started</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
+      <c r="F4" s="1" t="n">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1328561</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2460046</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>€2m - 7 Houses, Broadford</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Permitted – not started</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>46311</v>
       </c>
     </row>
   </sheetData>
@@ -3419,16 +3471,16 @@
         <v>2026</v>
       </c>
       <c r="B9" t="n">
-        <v>325</v>
+        <v>561</v>
       </c>
       <c r="C9" t="n">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="D9" t="n">
-        <v>156</v>
+        <v>306</v>
       </c>
       <c r="E9" t="n">
-        <v>119</v>
+        <v>179</v>
       </c>
       <c r="F9" t="n">
         <v>50</v>
@@ -3437,10 +3489,10 @@
         <v>270</v>
       </c>
       <c r="H9" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
       <c r="I9" t="n">
-        <v>1.31</v>
+        <v>0.71</v>
       </c>
     </row>
   </sheetData>
@@ -3881,16 +3933,16 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="K10" t="n">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="L10" t="n">
         <v>2</v>
       </c>
       <c r="M10" t="n">
-        <v>538</v>
+        <v>535</v>
       </c>
     </row>
   </sheetData>

</xml_diff>